<commit_message>
Fix: Isolate admin report errors in snapshot and add diagnostic logging
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21466243-053B-6C48-9718-0005C75F3104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D258E3D-6714-DC4C-ACEA-69B5465EB99A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="1340" yWindow="900" windowWidth="24460" windowHeight="16380" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -2211,7 +2211,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="1">
-        <v>46081</v>
+        <v>46092</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="46" thickBot="1" x14ac:dyDescent="0.25">
@@ -2284,49 +2284,49 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="15">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="B5" s="15">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C5" s="15">
-        <v>-40</v>
+        <v>-77</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.51282051282051277</v>
+        <v>-0.63114754098360648</v>
       </c>
       <c r="E5" s="15">
-        <v>3065.09</v>
+        <v>4684.3999999999996</v>
       </c>
       <c r="F5" s="15">
-        <v>1888.59</v>
+        <v>2468.83</v>
       </c>
       <c r="G5" s="15">
-        <v>-1176.5</v>
+        <v>-2215.5700000000002</v>
       </c>
       <c r="H5" s="16">
-        <v>-0.38383864747854068</v>
+        <v>-0.47296772265391507</v>
       </c>
       <c r="I5" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" s="15">
         <v>0</v>
       </c>
       <c r="K5" s="15">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="L5" s="16">
         <v>-1</v>
       </c>
       <c r="M5" s="15">
-        <v>141.97</v>
+        <v>313.24</v>
       </c>
       <c r="N5" s="15">
         <v>0</v>
       </c>
       <c r="O5" s="15">
-        <v>-141.97</v>
+        <v>-313.24</v>
       </c>
       <c r="P5" s="16">
         <v>-1</v>
@@ -2716,64 +2716,64 @@
         <v>128</v>
       </c>
       <c r="L7" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="11">
         <v>2</v>
       </c>
       <c r="N7" s="11">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="O7" s="12">
-        <v>-0.33329999999999999</v>
+        <v>-0.5</v>
       </c>
       <c r="P7" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q7" s="11">
         <v>2</v>
       </c>
       <c r="R7" s="11">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="S7" s="12">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="T7" s="11">
-        <v>25.07</v>
+        <v>134.32</v>
       </c>
       <c r="U7" s="11">
         <v>61.9</v>
       </c>
       <c r="V7" s="11">
-        <v>36.83</v>
+        <v>-72.42</v>
       </c>
       <c r="W7" s="12">
-        <v>1.4691000000000001</v>
+        <v>-0.53920000000000001</v>
       </c>
       <c r="X7" s="11">
-        <v>96.36</v>
+        <v>238.93</v>
       </c>
       <c r="Y7" s="11">
-        <v>112.49</v>
+        <v>115.62</v>
       </c>
       <c r="Z7" s="11">
-        <v>16.13</v>
+        <v>-123.31</v>
       </c>
       <c r="AA7" s="12">
-        <v>0.16739999999999999</v>
+        <v>-0.5161</v>
       </c>
       <c r="AB7" s="11">
-        <v>4.2222</v>
+        <v>5.3364000000000003</v>
       </c>
       <c r="AC7" s="11">
-        <v>5.1874000000000002</v>
+        <v>6.3615000000000004</v>
       </c>
       <c r="AD7" s="11">
-        <v>0.96519999999999995</v>
+        <v>1.0250999999999999</v>
       </c>
       <c r="AE7" s="12">
-        <v>0.2286</v>
+        <v>0.19209999999999999</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.2">
@@ -2847,13 +2847,13 @@
         <v>0</v>
       </c>
       <c r="X8" s="11">
-        <v>22.53</v>
+        <v>40.71</v>
       </c>
       <c r="Y8" s="11">
         <v>0</v>
       </c>
       <c r="Z8" s="11">
-        <v>-22.53</v>
+        <v>-40.71</v>
       </c>
       <c r="AA8" s="12">
         <v>-1</v>
@@ -2942,16 +2942,16 @@
         <v>-1</v>
       </c>
       <c r="X9" s="11">
-        <v>23.41</v>
+        <v>31.29</v>
       </c>
       <c r="Y9" s="11">
         <v>7.18</v>
       </c>
       <c r="Z9" s="11">
-        <v>-16.23</v>
+        <v>-24.11</v>
       </c>
       <c r="AA9" s="12">
-        <v>-0.69330000000000003</v>
+        <v>-0.77049999999999996</v>
       </c>
       <c r="AB9" s="11">
         <v>0</v>
@@ -3013,16 +3013,16 @@
         <v>-1</v>
       </c>
       <c r="P10" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="11">
         <v>0</v>
       </c>
       <c r="R10" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S10" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T10" s="11">
         <v>29.23</v>
@@ -3037,16 +3037,16 @@
         <v>-1</v>
       </c>
       <c r="X10" s="11">
-        <v>1.85</v>
+        <v>31.17</v>
       </c>
       <c r="Y10" s="11">
-        <v>2.75</v>
+        <v>5.51</v>
       </c>
       <c r="Z10" s="11">
-        <v>0.9</v>
+        <v>-25.66</v>
       </c>
       <c r="AA10" s="12">
-        <v>0.48649999999999999</v>
+        <v>-0.82320000000000004</v>
       </c>
       <c r="AB10" s="11">
         <v>0</v>
@@ -3132,13 +3132,13 @@
         <v>0</v>
       </c>
       <c r="X11" s="11">
-        <v>8.8699999999999992</v>
+        <v>13.32</v>
       </c>
       <c r="Y11" s="11">
         <v>0</v>
       </c>
       <c r="Z11" s="11">
-        <v>-8.8699999999999992</v>
+        <v>-13.32</v>
       </c>
       <c r="AA11" s="12">
         <v>-1</v>
@@ -3191,64 +3191,64 @@
         <v>128</v>
       </c>
       <c r="L12" s="11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M12" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="11">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="O12" s="12">
-        <v>-0.66669999999999996</v>
+        <v>-0.625</v>
       </c>
       <c r="P12" s="11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q12" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R12" s="11">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="S12" s="12">
-        <v>-0.66669999999999996</v>
+        <v>-0.625</v>
       </c>
       <c r="T12" s="11">
-        <v>149.66</v>
+        <v>279.27999999999997</v>
       </c>
       <c r="U12" s="11">
-        <v>44.67</v>
+        <v>75.27</v>
       </c>
       <c r="V12" s="11">
-        <v>-104.99</v>
+        <v>-204.01</v>
       </c>
       <c r="W12" s="12">
-        <v>-0.70150000000000001</v>
+        <v>-0.73050000000000004</v>
       </c>
       <c r="X12" s="11">
-        <v>415.45</v>
+        <v>574.09</v>
       </c>
       <c r="Y12" s="11">
-        <v>58.56</v>
+        <v>65.709999999999994</v>
       </c>
       <c r="Z12" s="11">
-        <v>-356.89</v>
+        <v>-508.38</v>
       </c>
       <c r="AA12" s="12">
-        <v>-0.85899999999999999</v>
+        <v>-0.88549999999999995</v>
       </c>
       <c r="AB12" s="11">
-        <v>2.6160999999999999</v>
+        <v>3.1593</v>
       </c>
       <c r="AC12" s="11">
-        <v>7.9966999999999997</v>
+        <v>17.5944</v>
       </c>
       <c r="AD12" s="11">
-        <v>5.3806000000000003</v>
+        <v>14.4351</v>
       </c>
       <c r="AE12" s="12">
-        <v>2.0567000000000002</v>
+        <v>4.5690999999999997</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
@@ -3322,28 +3322,28 @@
         <v>-1</v>
       </c>
       <c r="X13" s="11">
-        <v>74.97</v>
+        <v>99.88</v>
       </c>
       <c r="Y13" s="11">
-        <v>25.12</v>
+        <v>30.24</v>
       </c>
       <c r="Z13" s="11">
-        <v>-49.85</v>
+        <v>-69.64</v>
       </c>
       <c r="AA13" s="12">
-        <v>-0.66490000000000005</v>
+        <v>-0.69720000000000004</v>
       </c>
       <c r="AB13" s="11">
-        <v>5.8438999999999997</v>
+        <v>6.0643000000000002</v>
       </c>
       <c r="AC13" s="11">
-        <v>3.9805999999999999</v>
+        <v>4.0369999999999999</v>
       </c>
       <c r="AD13" s="11">
-        <v>-1.8633</v>
+        <v>-2.0272999999999999</v>
       </c>
       <c r="AE13" s="12">
-        <v>-0.31879999999999997</v>
+        <v>-0.33429999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
@@ -3417,13 +3417,13 @@
         <v>0</v>
       </c>
       <c r="X14" s="11">
-        <v>21.7</v>
+        <v>27.86</v>
       </c>
       <c r="Y14" s="11">
         <v>0</v>
       </c>
       <c r="Z14" s="11">
-        <v>-21.7</v>
+        <v>-27.86</v>
       </c>
       <c r="AA14" s="12">
         <v>-1</v>
@@ -3527,10 +3527,10 @@
         <v>0</v>
       </c>
       <c r="AC15" s="11">
-        <v>2.5028000000000001</v>
+        <v>3.2017000000000002</v>
       </c>
       <c r="AD15" s="11">
-        <v>2.5028000000000001</v>
+        <v>3.2017000000000002</v>
       </c>
       <c r="AE15" s="12">
         <v>1</v>
@@ -3669,61 +3669,61 @@
         <v>4</v>
       </c>
       <c r="M17" s="11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N17" s="11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="O17" s="12">
-        <v>-0.25</v>
+        <v>0.25</v>
       </c>
       <c r="P17" s="11">
         <v>6</v>
       </c>
       <c r="Q17" s="11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R17" s="11">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="S17" s="12">
-        <v>-0.5</v>
+        <v>-0.16669999999999999</v>
       </c>
       <c r="T17" s="11">
         <v>855.64</v>
       </c>
       <c r="U17" s="11">
-        <v>109.49</v>
+        <v>433.01</v>
       </c>
       <c r="V17" s="11">
-        <v>-746.15</v>
+        <v>-422.63</v>
       </c>
       <c r="W17" s="12">
-        <v>-0.872</v>
+        <v>-0.49390000000000001</v>
       </c>
       <c r="X17" s="11">
-        <v>571.64</v>
+        <v>588.49</v>
       </c>
       <c r="Y17" s="11">
-        <v>238.29</v>
+        <v>633.39</v>
       </c>
       <c r="Z17" s="11">
-        <v>-333.35</v>
+        <v>44.9</v>
       </c>
       <c r="AA17" s="12">
-        <v>-0.58309999999999995</v>
+        <v>7.6300000000000007E-2</v>
       </c>
       <c r="AB17" s="11">
-        <v>0.28599999999999998</v>
+        <v>0.69879999999999998</v>
       </c>
       <c r="AC17" s="11">
-        <v>0.74060000000000004</v>
+        <v>0.86550000000000005</v>
       </c>
       <c r="AD17" s="11">
-        <v>0.4546</v>
+        <v>0.16669999999999999</v>
       </c>
       <c r="AE17" s="12">
-        <v>1.5894999999999999</v>
+        <v>0.23860000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.2">
@@ -3797,28 +3797,28 @@
         <v>-1</v>
       </c>
       <c r="X18" s="11">
-        <v>22.54</v>
+        <v>25.91</v>
       </c>
       <c r="Y18" s="11">
-        <v>8.4</v>
+        <v>12.61</v>
       </c>
       <c r="Z18" s="11">
-        <v>-14.14</v>
+        <v>-13.3</v>
       </c>
       <c r="AA18" s="12">
-        <v>-0.62729999999999997</v>
+        <v>-0.51329999999999998</v>
       </c>
       <c r="AB18" s="11">
-        <v>0.81110000000000004</v>
+        <v>1.4147000000000001</v>
       </c>
       <c r="AC18" s="11">
-        <v>0.84189999999999998</v>
+        <v>1.4668000000000001</v>
       </c>
       <c r="AD18" s="11">
-        <v>3.0800000000000001E-2</v>
+        <v>5.21E-2</v>
       </c>
       <c r="AE18" s="12">
-        <v>3.7999999999999999E-2</v>
+        <v>3.6799999999999999E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.2">
@@ -3987,28 +3987,28 @@
         <v>-0.39219999999999999</v>
       </c>
       <c r="X20" s="11">
-        <v>259.25</v>
+        <v>353.8</v>
       </c>
       <c r="Y20" s="11">
         <v>202.83</v>
       </c>
       <c r="Z20" s="11">
-        <v>-56.42</v>
+        <v>-150.97</v>
       </c>
       <c r="AA20" s="12">
-        <v>-0.21759999999999999</v>
+        <v>-0.42670000000000002</v>
       </c>
       <c r="AB20" s="11">
-        <v>0.01</v>
+        <v>1.8688</v>
       </c>
       <c r="AC20" s="11">
-        <v>3.0000000000000001E-3</v>
+        <v>0.36919999999999997</v>
       </c>
       <c r="AD20" s="11">
-        <v>-7.0000000000000001E-3</v>
+        <v>-1.4996</v>
       </c>
       <c r="AE20" s="12">
-        <v>-0.7</v>
+        <v>-0.8024</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.2">
@@ -4082,28 +4082,28 @@
         <v>1</v>
       </c>
       <c r="X21" s="11">
-        <v>7.7</v>
+        <v>11.56</v>
       </c>
       <c r="Y21" s="11">
         <v>59.85</v>
       </c>
       <c r="Z21" s="11">
-        <v>52.15</v>
+        <v>48.29</v>
       </c>
       <c r="AA21" s="12">
-        <v>6.7727000000000004</v>
+        <v>4.1772999999999998</v>
       </c>
       <c r="AB21" s="11">
-        <v>0.20960000000000001</v>
+        <v>0.31490000000000001</v>
       </c>
       <c r="AC21" s="11">
-        <v>0.7792</v>
+        <v>1.1247</v>
       </c>
       <c r="AD21" s="11">
-        <v>0.5696</v>
+        <v>0.80979999999999996</v>
       </c>
       <c r="AE21" s="12">
-        <v>2.7176</v>
+        <v>2.5716000000000001</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.2">
@@ -4180,13 +4180,13 @@
         <v>11.23</v>
       </c>
       <c r="Y22" s="11">
-        <v>0</v>
+        <v>10.14</v>
       </c>
       <c r="Z22" s="11">
-        <v>-11.23</v>
+        <v>-1.0900000000000001</v>
       </c>
       <c r="AA22" s="12">
-        <v>-1</v>
+        <v>-9.7100000000000006E-2</v>
       </c>
       <c r="AB22" s="11">
         <v>0</v>
@@ -4236,52 +4236,52 @@
         <v>128</v>
       </c>
       <c r="L23" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M23" s="11">
         <v>1</v>
       </c>
       <c r="N23" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O23" s="12">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="P23" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q23" s="11">
         <v>1</v>
       </c>
       <c r="R23" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S23" s="12">
-        <v>0</v>
+        <v>-0.5</v>
       </c>
       <c r="T23" s="11">
-        <v>45.49</v>
+        <v>72.900000000000006</v>
       </c>
       <c r="U23" s="11">
         <v>46.1</v>
       </c>
       <c r="V23" s="11">
-        <v>0.61</v>
+        <v>-26.8</v>
       </c>
       <c r="W23" s="12">
-        <v>1.34E-2</v>
+        <v>-0.36759999999999998</v>
       </c>
       <c r="X23" s="11">
-        <v>5.81</v>
+        <v>11.9</v>
       </c>
       <c r="Y23" s="11">
         <v>16.34</v>
       </c>
       <c r="Z23" s="11">
-        <v>10.53</v>
+        <v>4.4400000000000004</v>
       </c>
       <c r="AA23" s="12">
-        <v>1.8124</v>
+        <v>0.37309999999999999</v>
       </c>
       <c r="AB23" s="11">
         <v>0</v>
@@ -4367,13 +4367,13 @@
         <v>0</v>
       </c>
       <c r="X24" s="11">
-        <v>5.42</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="Y24" s="11">
         <v>0</v>
       </c>
       <c r="Z24" s="11">
-        <v>-5.42</v>
+        <v>-8.3800000000000008</v>
       </c>
       <c r="AA24" s="12">
         <v>-1</v>
@@ -4462,13 +4462,13 @@
         <v>0</v>
       </c>
       <c r="X25" s="11">
-        <v>2.2000000000000002</v>
+        <v>4.42</v>
       </c>
       <c r="Y25" s="11">
         <v>0</v>
       </c>
       <c r="Z25" s="11">
-        <v>-2.2000000000000002</v>
+        <v>-4.42</v>
       </c>
       <c r="AA25" s="12">
         <v>-1</v>
@@ -4557,16 +4557,16 @@
         <v>-0.58879999999999999</v>
       </c>
       <c r="X26" s="11">
-        <v>64.19</v>
+        <v>78.84</v>
       </c>
       <c r="Y26" s="11">
-        <v>42.45</v>
+        <v>46.37</v>
       </c>
       <c r="Z26" s="11">
-        <v>-21.74</v>
+        <v>-32.47</v>
       </c>
       <c r="AA26" s="12">
-        <v>-0.3387</v>
+        <v>-0.4118</v>
       </c>
       <c r="AB26" s="11">
         <v>0.5141</v>
@@ -4628,40 +4628,40 @@
         <v>-1</v>
       </c>
       <c r="P27" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q27" s="11">
         <v>0</v>
       </c>
       <c r="R27" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S27" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T27" s="11">
-        <v>39.299999999999997</v>
+        <v>9.4</v>
       </c>
       <c r="U27" s="11">
         <v>0</v>
       </c>
       <c r="V27" s="11">
-        <v>-39.299999999999997</v>
+        <v>-9.4</v>
       </c>
       <c r="W27" s="12">
         <v>-1</v>
       </c>
       <c r="X27" s="11">
-        <v>23.02</v>
+        <v>46.3</v>
       </c>
       <c r="Y27" s="11">
-        <v>17.43</v>
+        <v>19.75</v>
       </c>
       <c r="Z27" s="11">
-        <v>-5.59</v>
+        <v>-26.55</v>
       </c>
       <c r="AA27" s="12">
-        <v>-0.24279999999999999</v>
+        <v>-0.57340000000000002</v>
       </c>
       <c r="AB27" s="11">
         <v>0</v>
@@ -4747,16 +4747,16 @@
         <v>0</v>
       </c>
       <c r="X28" s="11">
-        <v>1.54</v>
+        <v>3.09</v>
       </c>
       <c r="Y28" s="11">
-        <v>9.73</v>
+        <v>11.47</v>
       </c>
       <c r="Z28" s="11">
-        <v>8.19</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="AA28" s="12">
-        <v>5.3182</v>
+        <v>2.7120000000000002</v>
       </c>
       <c r="AB28" s="11">
         <v>0</v>
@@ -4806,64 +4806,64 @@
         <v>131</v>
       </c>
       <c r="L29" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M29" s="11">
         <v>0</v>
       </c>
       <c r="N29" s="11">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="O29" s="12">
         <v>-1</v>
       </c>
       <c r="P29" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q29" s="11">
         <v>0</v>
       </c>
       <c r="R29" s="11">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="S29" s="12">
         <v>-1</v>
       </c>
       <c r="T29" s="11">
-        <v>93.83</v>
+        <v>175.1</v>
       </c>
       <c r="U29" s="11">
         <v>0</v>
       </c>
       <c r="V29" s="11">
-        <v>-93.83</v>
+        <v>-175.1</v>
       </c>
       <c r="W29" s="12">
         <v>-1</v>
       </c>
       <c r="X29" s="11">
-        <v>94.31</v>
+        <v>215.39</v>
       </c>
       <c r="Y29" s="11">
-        <v>24.18</v>
+        <v>28.61</v>
       </c>
       <c r="Z29" s="11">
-        <v>-70.13</v>
+        <v>-186.78</v>
       </c>
       <c r="AA29" s="12">
-        <v>-0.74360000000000004</v>
+        <v>-0.86719999999999997</v>
       </c>
       <c r="AB29" s="11">
-        <v>0.15720000000000001</v>
+        <v>1.528</v>
       </c>
       <c r="AC29" s="11">
-        <v>1.5749</v>
+        <v>2.7492999999999999</v>
       </c>
       <c r="AD29" s="11">
-        <v>1.4177</v>
+        <v>1.2213000000000001</v>
       </c>
       <c r="AE29" s="12">
-        <v>9.0183999999999997</v>
+        <v>0.79930000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.2">
@@ -4901,64 +4901,64 @@
         <v>131</v>
       </c>
       <c r="L30" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M30" s="11">
         <v>3</v>
       </c>
       <c r="N30" s="11">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="O30" s="12">
-        <v>-0.25</v>
+        <v>-0.625</v>
       </c>
       <c r="P30" s="11">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q30" s="11">
         <v>3</v>
       </c>
       <c r="R30" s="11">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="S30" s="12">
-        <v>-0.25</v>
+        <v>-0.57140000000000002</v>
       </c>
       <c r="T30" s="11">
-        <v>107.55</v>
+        <v>224.88</v>
       </c>
       <c r="U30" s="11">
         <v>86.32</v>
       </c>
       <c r="V30" s="11">
-        <v>-21.23</v>
+        <v>-138.56</v>
       </c>
       <c r="W30" s="12">
-        <v>-0.19739999999999999</v>
+        <v>-0.61619999999999997</v>
       </c>
       <c r="X30" s="11">
-        <v>109.35</v>
+        <v>227.28</v>
       </c>
       <c r="Y30" s="11">
-        <v>67.709999999999994</v>
+        <v>79.98</v>
       </c>
       <c r="Z30" s="11">
-        <v>-41.64</v>
+        <v>-147.30000000000001</v>
       </c>
       <c r="AA30" s="12">
-        <v>-0.38080000000000003</v>
+        <v>-0.64810000000000001</v>
       </c>
       <c r="AB30" s="11">
-        <v>3.8600000000000002E-2</v>
+        <v>0.1235</v>
       </c>
       <c r="AC30" s="11">
         <v>0.56420000000000003</v>
       </c>
       <c r="AD30" s="11">
-        <v>0.52559999999999996</v>
+        <v>0.44069999999999998</v>
       </c>
       <c r="AE30" s="12">
-        <v>13.6166</v>
+        <v>3.5684</v>
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.2">
@@ -4996,64 +4996,64 @@
         <v>131</v>
       </c>
       <c r="L31" s="11">
+        <v>7</v>
+      </c>
+      <c r="M31" s="11">
         <v>3</v>
       </c>
-      <c r="M31" s="11">
-        <v>2</v>
-      </c>
       <c r="N31" s="11">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="O31" s="12">
-        <v>-0.33329999999999999</v>
+        <v>-0.57140000000000002</v>
       </c>
       <c r="P31" s="11">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="Q31" s="11">
         <v>3</v>
       </c>
       <c r="R31" s="11">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="S31" s="12">
-        <v>0</v>
+        <v>-0.57140000000000002</v>
       </c>
       <c r="T31" s="11">
-        <v>121.6</v>
+        <v>212.51</v>
       </c>
       <c r="U31" s="11">
-        <v>44.05</v>
+        <v>68.92</v>
       </c>
       <c r="V31" s="11">
-        <v>-77.55</v>
+        <v>-143.59</v>
       </c>
       <c r="W31" s="12">
-        <v>-0.63770000000000004</v>
+        <v>-0.67569999999999997</v>
       </c>
       <c r="X31" s="11">
-        <v>121.85</v>
+        <v>187.2</v>
       </c>
       <c r="Y31" s="11">
-        <v>49.24</v>
+        <v>58.89</v>
       </c>
       <c r="Z31" s="11">
-        <v>-72.61</v>
+        <v>-128.31</v>
       </c>
       <c r="AA31" s="12">
-        <v>-0.59589999999999999</v>
+        <v>-0.68540000000000001</v>
       </c>
       <c r="AB31" s="11">
-        <v>0.35880000000000001</v>
+        <v>0.79920000000000002</v>
       </c>
       <c r="AC31" s="11">
-        <v>0.72289999999999999</v>
+        <v>1.1778999999999999</v>
       </c>
       <c r="AD31" s="11">
-        <v>0.36409999999999998</v>
+        <v>0.37869999999999998</v>
       </c>
       <c r="AE31" s="12">
-        <v>1.0147999999999999</v>
+        <v>0.4738</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.2">
@@ -5091,52 +5091,52 @@
         <v>131</v>
       </c>
       <c r="L32" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M32" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N32" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O32" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q32" s="11">
         <v>1</v>
       </c>
       <c r="R32" s="11">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="S32" s="12">
-        <v>1</v>
+        <v>-0.5</v>
       </c>
       <c r="T32" s="11">
-        <v>0</v>
+        <v>49.3</v>
       </c>
       <c r="U32" s="11">
-        <v>30.84</v>
+        <v>61.31</v>
       </c>
       <c r="V32" s="11">
-        <v>30.84</v>
+        <v>12.01</v>
       </c>
       <c r="W32" s="12">
-        <v>1</v>
+        <v>0.24360000000000001</v>
       </c>
       <c r="X32" s="11">
-        <v>20.77</v>
+        <v>80.510000000000005</v>
       </c>
       <c r="Y32" s="11">
-        <v>24.37</v>
+        <v>26.09</v>
       </c>
       <c r="Z32" s="11">
-        <v>3.6</v>
+        <v>-54.42</v>
       </c>
       <c r="AA32" s="12">
-        <v>0.17330000000000001</v>
+        <v>-0.67589999999999995</v>
       </c>
       <c r="AB32" s="11">
         <v>0</v>
@@ -5186,64 +5186,64 @@
         <v>127</v>
       </c>
       <c r="L33" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M33" s="11">
         <v>0</v>
       </c>
       <c r="N33" s="11">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="O33" s="12">
         <v>-1</v>
       </c>
       <c r="P33" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q33" s="11">
         <v>0</v>
       </c>
       <c r="R33" s="11">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="S33" s="12">
         <v>-1</v>
       </c>
       <c r="T33" s="11">
-        <v>49.01</v>
+        <v>67.260000000000005</v>
       </c>
       <c r="U33" s="11">
         <v>0</v>
       </c>
       <c r="V33" s="11">
-        <v>-49.01</v>
+        <v>-67.260000000000005</v>
       </c>
       <c r="W33" s="12">
         <v>-1</v>
       </c>
       <c r="X33" s="11">
-        <v>54.74</v>
+        <v>73</v>
       </c>
       <c r="Y33" s="11">
-        <v>19.7</v>
+        <v>22.78</v>
       </c>
       <c r="Z33" s="11">
-        <v>-35.04</v>
+        <v>-50.22</v>
       </c>
       <c r="AA33" s="12">
-        <v>-0.6401</v>
+        <v>-0.68789999999999996</v>
       </c>
       <c r="AB33" s="11">
-        <v>3.1772999999999998</v>
+        <v>3.1848999999999998</v>
       </c>
       <c r="AC33" s="11">
         <v>0.71109999999999995</v>
       </c>
       <c r="AD33" s="11">
-        <v>-2.4662000000000002</v>
+        <v>-2.4738000000000002</v>
       </c>
       <c r="AE33" s="12">
-        <v>-0.7762</v>
+        <v>-0.77669999999999995</v>
       </c>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.2">
@@ -5281,52 +5281,52 @@
         <v>127</v>
       </c>
       <c r="L34" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M34" s="11">
         <v>1</v>
       </c>
       <c r="N34" s="11">
-        <v>-3</v>
+        <v>-7</v>
       </c>
       <c r="O34" s="12">
-        <v>-0.75</v>
+        <v>-0.875</v>
       </c>
       <c r="P34" s="11">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q34" s="11">
         <v>0</v>
       </c>
       <c r="R34" s="11">
-        <v>-1</v>
+        <v>-6</v>
       </c>
       <c r="S34" s="12">
         <v>-1</v>
       </c>
       <c r="T34" s="11">
-        <v>191.52</v>
+        <v>406.35</v>
       </c>
       <c r="U34" s="11">
         <v>-1319.02</v>
       </c>
       <c r="V34" s="11">
-        <v>-1510.54</v>
+        <v>-1725.37</v>
       </c>
       <c r="W34" s="12">
-        <v>-7.8871000000000002</v>
+        <v>-4.2460000000000004</v>
       </c>
       <c r="X34" s="11">
-        <v>25.02</v>
+        <v>63.59</v>
       </c>
       <c r="Y34" s="11">
-        <v>66.02</v>
+        <v>72.59</v>
       </c>
       <c r="Z34" s="11">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="AA34" s="12">
-        <v>1.6387</v>
+        <v>0.14149999999999999</v>
       </c>
       <c r="AB34" s="11">
         <v>0</v>
@@ -5471,64 +5471,64 @@
         <v>127</v>
       </c>
       <c r="L36" s="11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M36" s="11">
         <v>1</v>
       </c>
       <c r="N36" s="11">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="O36" s="12">
-        <v>-0.83330000000000004</v>
+        <v>-0.85709999999999997</v>
       </c>
       <c r="P36" s="11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q36" s="11">
         <v>1</v>
       </c>
       <c r="R36" s="11">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="S36" s="12">
-        <v>-0.8</v>
+        <v>-0.83330000000000004</v>
       </c>
       <c r="T36" s="11">
-        <v>203.63</v>
+        <v>223.13</v>
       </c>
       <c r="U36" s="11">
         <v>36.93</v>
       </c>
       <c r="V36" s="11">
-        <v>-166.7</v>
+        <v>-186.2</v>
       </c>
       <c r="W36" s="12">
-        <v>-0.81859999999999999</v>
+        <v>-0.83450000000000002</v>
       </c>
       <c r="X36" s="11">
-        <v>250.75</v>
+        <v>303.52999999999997</v>
       </c>
       <c r="Y36" s="11">
-        <v>59.09</v>
+        <v>64.94</v>
       </c>
       <c r="Z36" s="11">
-        <v>-191.66</v>
+        <v>-238.59</v>
       </c>
       <c r="AA36" s="12">
-        <v>-0.76429999999999998</v>
+        <v>-0.78610000000000002</v>
       </c>
       <c r="AB36" s="11">
-        <v>2.6915</v>
+        <v>4.0427</v>
       </c>
       <c r="AC36" s="11">
         <v>2.7980999999999998</v>
       </c>
       <c r="AD36" s="11">
-        <v>0.1066</v>
+        <v>-1.2445999999999999</v>
       </c>
       <c r="AE36" s="12">
-        <v>3.9600000000000003E-2</v>
+        <v>-0.30790000000000001</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.2">
@@ -5566,52 +5566,52 @@
         <v>127</v>
       </c>
       <c r="L37" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M37" s="11">
         <v>1</v>
       </c>
       <c r="N37" s="11">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="O37" s="12">
-        <v>-0.75</v>
+        <v>-0.8</v>
       </c>
       <c r="P37" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q37" s="11">
         <v>1</v>
       </c>
       <c r="R37" s="11">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="S37" s="12">
-        <v>-0.75</v>
+        <v>-0.8</v>
       </c>
       <c r="T37" s="11">
-        <v>114.51</v>
+        <v>149.02000000000001</v>
       </c>
       <c r="U37" s="11">
         <v>36.159999999999997</v>
       </c>
       <c r="V37" s="11">
-        <v>-78.349999999999994</v>
+        <v>-112.86</v>
       </c>
       <c r="W37" s="12">
-        <v>-0.68420000000000003</v>
+        <v>-0.75729999999999997</v>
       </c>
       <c r="X37" s="11">
-        <v>53.59</v>
+        <v>86.18</v>
       </c>
       <c r="Y37" s="11">
-        <v>112.26</v>
+        <v>119.74</v>
       </c>
       <c r="Z37" s="11">
-        <v>58.67</v>
+        <v>33.56</v>
       </c>
       <c r="AA37" s="12">
-        <v>1.0948</v>
+        <v>0.38940000000000002</v>
       </c>
       <c r="AB37" s="11">
         <v>0</v>
@@ -5661,61 +5661,61 @@
         <v>127</v>
       </c>
       <c r="L38" s="11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M38" s="11">
         <v>0</v>
       </c>
       <c r="N38" s="11">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="O38" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P38" s="11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q38" s="11">
         <v>0</v>
       </c>
       <c r="R38" s="11">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="S38" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T38" s="11">
-        <v>0</v>
+        <v>90.67</v>
       </c>
       <c r="U38" s="11">
         <v>0</v>
       </c>
       <c r="V38" s="11">
-        <v>0</v>
+        <v>-90.67</v>
       </c>
       <c r="W38" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X38" s="11">
-        <v>42.18</v>
+        <v>103.45</v>
       </c>
       <c r="Y38" s="11">
         <v>8.83</v>
       </c>
       <c r="Z38" s="11">
-        <v>-33.35</v>
+        <v>-94.62</v>
       </c>
       <c r="AA38" s="12">
-        <v>-0.79069999999999996</v>
+        <v>-0.91459999999999997</v>
       </c>
       <c r="AB38" s="11">
-        <v>8.9999999999999998E-4</v>
+        <v>3.3999999999999998E-3</v>
       </c>
       <c r="AC38" s="11">
         <v>0</v>
       </c>
       <c r="AD38" s="11">
-        <v>-8.9999999999999998E-4</v>
+        <v>-3.3999999999999998E-3</v>
       </c>
       <c r="AE38" s="12">
         <v>-1</v>
@@ -5768,13 +5768,13 @@
         <v>-1</v>
       </c>
       <c r="P39" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q39" s="11">
         <v>0</v>
       </c>
       <c r="R39" s="11">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="S39" s="12">
         <v>-1</v>
@@ -5792,28 +5792,28 @@
         <v>-1</v>
       </c>
       <c r="X39" s="11">
-        <v>19.489999999999998</v>
+        <v>44.5</v>
       </c>
       <c r="Y39" s="11">
         <v>0</v>
       </c>
       <c r="Z39" s="11">
-        <v>-19.489999999999998</v>
+        <v>-44.5</v>
       </c>
       <c r="AA39" s="12">
         <v>-1</v>
       </c>
       <c r="AB39" s="11">
-        <v>0</v>
+        <v>9.8100000000000007E-2</v>
       </c>
       <c r="AC39" s="11">
         <v>0</v>
       </c>
       <c r="AD39" s="11">
-        <v>0</v>
+        <v>-9.8100000000000007E-2</v>
       </c>
       <c r="AE39" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.2">
@@ -5887,16 +5887,16 @@
         <v>-1</v>
       </c>
       <c r="X40" s="11">
-        <v>18.02</v>
+        <v>29.29</v>
       </c>
       <c r="Y40" s="11">
-        <v>15.96</v>
+        <v>16.809999999999999</v>
       </c>
       <c r="Z40" s="11">
-        <v>-2.06</v>
+        <v>-12.48</v>
       </c>
       <c r="AA40" s="12">
-        <v>-0.1143</v>
+        <v>-0.42609999999999998</v>
       </c>
       <c r="AB40" s="11">
         <v>0</v>
@@ -5982,13 +5982,13 @@
         <v>0</v>
       </c>
       <c r="X41" s="11">
-        <v>2.97</v>
+        <v>4.46</v>
       </c>
       <c r="Y41" s="11">
         <v>0</v>
       </c>
       <c r="Z41" s="11">
-        <v>-2.97</v>
+        <v>-4.46</v>
       </c>
       <c r="AA41" s="12">
         <v>-1</v>
@@ -6041,49 +6041,49 @@
         <v>127</v>
       </c>
       <c r="L42" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M42" s="11">
         <v>0</v>
       </c>
       <c r="N42" s="11">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="O42" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P42" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q42" s="11">
         <v>0</v>
       </c>
       <c r="R42" s="11">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="S42" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T42" s="11">
-        <v>0</v>
+        <v>97.1</v>
       </c>
       <c r="U42" s="11">
         <v>0</v>
       </c>
       <c r="V42" s="11">
-        <v>0</v>
+        <v>-97.1</v>
       </c>
       <c r="W42" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X42" s="11">
-        <v>19.25</v>
+        <v>140.68</v>
       </c>
       <c r="Y42" s="11">
         <v>0</v>
       </c>
       <c r="Z42" s="11">
-        <v>-19.25</v>
+        <v>-140.68</v>
       </c>
       <c r="AA42" s="12">
         <v>-1</v>
@@ -6160,28 +6160,28 @@
         <v>-1</v>
       </c>
       <c r="T43" s="11">
-        <v>-3.19</v>
+        <v>-35.53</v>
       </c>
       <c r="U43" s="11">
         <v>28.7</v>
       </c>
       <c r="V43" s="11">
-        <v>31.89</v>
+        <v>64.23</v>
       </c>
       <c r="W43" s="12">
-        <v>9.9969000000000001</v>
+        <v>1.8078000000000001</v>
       </c>
       <c r="X43" s="11">
-        <v>52.34</v>
+        <v>62.03</v>
       </c>
       <c r="Y43" s="11">
         <v>5.68</v>
       </c>
       <c r="Z43" s="11">
-        <v>-46.66</v>
+        <v>-56.35</v>
       </c>
       <c r="AA43" s="12">
-        <v>-0.89149999999999996</v>
+        <v>-0.90839999999999999</v>
       </c>
       <c r="AB43" s="11">
         <v>0</v>
@@ -6231,52 +6231,52 @@
         <v>127</v>
       </c>
       <c r="L44" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M44" s="11">
         <v>0</v>
       </c>
       <c r="N44" s="11">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="O44" s="12">
         <v>-1</v>
       </c>
       <c r="P44" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q44" s="11">
         <v>0</v>
       </c>
       <c r="R44" s="11">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="S44" s="12">
         <v>-1</v>
       </c>
       <c r="T44" s="11">
-        <v>30.34</v>
+        <v>50.61</v>
       </c>
       <c r="U44" s="11">
         <v>0</v>
       </c>
       <c r="V44" s="11">
-        <v>-30.34</v>
+        <v>-50.61</v>
       </c>
       <c r="W44" s="12">
         <v>-1</v>
       </c>
       <c r="X44" s="11">
-        <v>34.43</v>
+        <v>44.35</v>
       </c>
       <c r="Y44" s="11">
         <v>17.68</v>
       </c>
       <c r="Z44" s="11">
-        <v>-16.75</v>
+        <v>-26.67</v>
       </c>
       <c r="AA44" s="12">
-        <v>-0.48649999999999999</v>
+        <v>-0.60140000000000005</v>
       </c>
       <c r="AB44" s="11">
         <v>0</v>
@@ -6326,64 +6326,64 @@
         <v>127</v>
       </c>
       <c r="L45" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="M45" s="11">
+        <v>7</v>
+      </c>
+      <c r="N45" s="11">
+        <v>-5</v>
+      </c>
+      <c r="O45" s="12">
+        <v>-0.41670000000000001</v>
+      </c>
+      <c r="P45" s="11">
+        <v>12</v>
+      </c>
+      <c r="Q45" s="11">
         <v>6</v>
       </c>
-      <c r="N45" s="11">
-        <v>-3</v>
-      </c>
-      <c r="O45" s="12">
-        <v>-0.33329999999999999</v>
-      </c>
-      <c r="P45" s="11">
-        <v>9</v>
-      </c>
-      <c r="Q45" s="11">
-        <v>5</v>
-      </c>
       <c r="R45" s="11">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="S45" s="12">
-        <v>-0.44440000000000002</v>
+        <v>-0.5</v>
       </c>
       <c r="T45" s="11">
-        <v>219.18</v>
+        <v>272.62</v>
       </c>
       <c r="U45" s="11">
-        <v>181.35</v>
+        <v>227.64</v>
       </c>
       <c r="V45" s="11">
-        <v>-37.83</v>
+        <v>-44.98</v>
       </c>
       <c r="W45" s="12">
-        <v>-0.1726</v>
+        <v>-0.16500000000000001</v>
       </c>
       <c r="X45" s="11">
-        <v>129.72</v>
+        <v>156.13999999999999</v>
       </c>
       <c r="Y45" s="11">
-        <v>89.24</v>
+        <v>144.81</v>
       </c>
       <c r="Z45" s="11">
-        <v>-40.479999999999997</v>
+        <v>-11.33</v>
       </c>
       <c r="AA45" s="12">
-        <v>-0.31209999999999999</v>
+        <v>-7.2599999999999998E-2</v>
       </c>
       <c r="AB45" s="11">
         <v>0.2029</v>
       </c>
       <c r="AC45" s="11">
-        <v>0.30380000000000001</v>
+        <v>0.4355</v>
       </c>
       <c r="AD45" s="11">
-        <v>0.1009</v>
+        <v>0.2326</v>
       </c>
       <c r="AE45" s="12">
-        <v>0.49730000000000002</v>
+        <v>1.1464000000000001</v>
       </c>
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.2">
@@ -6457,16 +6457,16 @@
         <v>-1</v>
       </c>
       <c r="X46" s="11">
-        <v>140.16</v>
+        <v>208.83</v>
       </c>
       <c r="Y46" s="11">
         <v>28.49</v>
       </c>
       <c r="Z46" s="11">
-        <v>-111.67</v>
+        <v>-180.34</v>
       </c>
       <c r="AA46" s="12">
-        <v>-0.79669999999999996</v>
+        <v>-0.86360000000000003</v>
       </c>
       <c r="AB46" s="11">
         <v>0</v>
@@ -6552,13 +6552,13 @@
         <v>0</v>
       </c>
       <c r="X47" s="11">
-        <v>6.2</v>
+        <v>9.74</v>
       </c>
       <c r="Y47" s="11">
         <v>0</v>
       </c>
       <c r="Z47" s="11">
-        <v>-6.2</v>
+        <v>-9.74</v>
       </c>
       <c r="AA47" s="12">
         <v>-1</v>
@@ -6611,52 +6611,52 @@
         <v>127</v>
       </c>
       <c r="L48" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M48" s="11">
         <v>0</v>
       </c>
       <c r="N48" s="11">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="O48" s="12">
         <v>-1</v>
       </c>
       <c r="P48" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q48" s="11">
         <v>0</v>
       </c>
       <c r="R48" s="11">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="S48" s="12">
         <v>-1</v>
       </c>
       <c r="T48" s="11">
-        <v>106.85</v>
+        <v>169.31</v>
       </c>
       <c r="U48" s="11">
         <v>0</v>
       </c>
       <c r="V48" s="11">
-        <v>-106.85</v>
+        <v>-169.31</v>
       </c>
       <c r="W48" s="12">
         <v>-1</v>
       </c>
       <c r="X48" s="11">
-        <v>16.75</v>
+        <v>86.46</v>
       </c>
       <c r="Y48" s="11">
-        <v>23.01</v>
+        <v>28.41</v>
       </c>
       <c r="Z48" s="11">
-        <v>6.26</v>
+        <v>-58.05</v>
       </c>
       <c r="AA48" s="12">
-        <v>0.37369999999999998</v>
+        <v>-0.6714</v>
       </c>
       <c r="AB48" s="11">
         <v>0</v>
@@ -6706,52 +6706,52 @@
         <v>132</v>
       </c>
       <c r="L49" s="11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M49" s="11">
         <v>0</v>
       </c>
       <c r="N49" s="11">
-        <v>-3</v>
+        <v>-6</v>
       </c>
       <c r="O49" s="12">
         <v>-1</v>
       </c>
       <c r="P49" s="11">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="Q49" s="11">
         <v>0</v>
       </c>
       <c r="R49" s="11">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="S49" s="12">
         <v>-1</v>
       </c>
       <c r="T49" s="11">
-        <v>142.29</v>
+        <v>228.19</v>
       </c>
       <c r="U49" s="11">
         <v>0</v>
       </c>
       <c r="V49" s="11">
-        <v>-142.29</v>
+        <v>-228.19</v>
       </c>
       <c r="W49" s="12">
         <v>-1</v>
       </c>
       <c r="X49" s="11">
-        <v>141.97</v>
+        <v>181.68</v>
       </c>
       <c r="Y49" s="11">
         <v>13.5</v>
       </c>
       <c r="Z49" s="11">
-        <v>-128.47</v>
+        <v>-168.18</v>
       </c>
       <c r="AA49" s="12">
-        <v>-0.90490000000000004</v>
+        <v>-0.92569999999999997</v>
       </c>
       <c r="AB49" s="11">
         <v>0</v>
@@ -6789,7 +6789,7 @@
         <v>60</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I50" s="22">
         <v>45736</v>
@@ -6801,49 +6801,49 @@
         <v>132</v>
       </c>
       <c r="L50" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M50" s="11">
         <v>0</v>
       </c>
       <c r="N50" s="11">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="O50" s="12">
         <v>-1</v>
       </c>
       <c r="P50" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q50" s="11">
         <v>0</v>
       </c>
       <c r="R50" s="11">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="S50" s="12">
         <v>-1</v>
       </c>
       <c r="T50" s="11">
-        <v>44.44</v>
+        <v>133.03</v>
       </c>
       <c r="U50" s="11">
         <v>0</v>
       </c>
       <c r="V50" s="11">
-        <v>-44.44</v>
+        <v>-133.03</v>
       </c>
       <c r="W50" s="12">
         <v>-1</v>
       </c>
       <c r="X50" s="11">
-        <v>44.44</v>
+        <v>131.56</v>
       </c>
       <c r="Y50" s="11">
         <v>0</v>
       </c>
       <c r="Z50" s="11">
-        <v>-44.44</v>
+        <v>-131.56</v>
       </c>
       <c r="AA50" s="12">
         <v>-1</v>
@@ -6991,52 +6991,52 @@
         <v>132</v>
       </c>
       <c r="L52" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M52" s="11">
         <v>0</v>
       </c>
       <c r="N52" s="11">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="O52" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P52" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q52" s="11">
         <v>0</v>
       </c>
       <c r="R52" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S52" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T52" s="11">
-        <v>0</v>
+        <v>53.09</v>
       </c>
       <c r="U52" s="11">
         <v>0</v>
       </c>
       <c r="V52" s="11">
-        <v>0</v>
+        <v>-53.09</v>
       </c>
       <c r="W52" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X52" s="11">
-        <v>0</v>
+        <v>2.4500000000000002</v>
       </c>
       <c r="Y52" s="11">
         <v>13.31</v>
       </c>
       <c r="Z52" s="11">
-        <v>13.31</v>
+        <v>10.86</v>
       </c>
       <c r="AA52" s="12">
-        <v>1</v>
+        <v>4.4326999999999996</v>
       </c>
       <c r="AB52" s="11">
         <v>0</v>
@@ -7086,52 +7086,52 @@
         <v>132</v>
       </c>
       <c r="L53" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M53" s="11">
         <v>0</v>
       </c>
       <c r="N53" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="O53" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="P53" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q53" s="11">
         <v>0</v>
       </c>
       <c r="R53" s="11">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="S53" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T53" s="11">
-        <v>0</v>
+        <v>27.65</v>
       </c>
       <c r="U53" s="11">
         <v>0</v>
       </c>
       <c r="V53" s="11">
-        <v>0</v>
+        <v>-27.65</v>
       </c>
       <c r="W53" s="12">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="X53" s="11">
-        <v>0</v>
+        <v>13.82</v>
       </c>
       <c r="Y53" s="11">
-        <v>13.16</v>
+        <v>17.690000000000001</v>
       </c>
       <c r="Z53" s="11">
-        <v>13.16</v>
+        <v>3.87</v>
       </c>
       <c r="AA53" s="12">
-        <v>1</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="AB53" s="11">
         <v>0</v>
@@ -7220,10 +7220,10 @@
         <v>0</v>
       </c>
       <c r="Y54" s="11">
-        <v>84.11</v>
+        <v>67.709999999999994</v>
       </c>
       <c r="Z54" s="11">
-        <v>84.11</v>
+        <v>67.709999999999994</v>
       </c>
       <c r="AA54" s="12">
         <v>1</v>
@@ -7315,10 +7315,10 @@
         <v>0</v>
       </c>
       <c r="Y55" s="11">
-        <v>37.08</v>
+        <v>39.47</v>
       </c>
       <c r="Z55" s="11">
-        <v>37.08</v>
+        <v>39.47</v>
       </c>
       <c r="AA55" s="12">
         <v>1</v>
@@ -7410,10 +7410,10 @@
         <v>0</v>
       </c>
       <c r="Y56" s="11">
-        <v>10.48</v>
+        <v>15.97</v>
       </c>
       <c r="Z56" s="11">
-        <v>10.48</v>
+        <v>15.97</v>
       </c>
       <c r="AA56" s="12">
         <v>1</v>
@@ -7659,10 +7659,10 @@
         <v>0</v>
       </c>
       <c r="M59" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N59" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O59" s="12">
         <v>1</v>
@@ -7683,10 +7683,10 @@
         <v>0</v>
       </c>
       <c r="U59" s="11">
-        <v>51.35</v>
+        <v>75.849999999999994</v>
       </c>
       <c r="V59" s="11">
-        <v>51.35</v>
+        <v>75.849999999999994</v>
       </c>
       <c r="W59" s="12">
         <v>1</v>
@@ -7695,10 +7695,10 @@
         <v>0</v>
       </c>
       <c r="Y59" s="11">
-        <v>90.8</v>
+        <v>110.56</v>
       </c>
       <c r="Z59" s="11">
-        <v>90.8</v>
+        <v>110.56</v>
       </c>
       <c r="AA59" s="12">
         <v>1</v>
@@ -7707,10 +7707,10 @@
         <v>0</v>
       </c>
       <c r="AC59" s="11">
-        <v>0.46429999999999999</v>
+        <v>1.1674</v>
       </c>
       <c r="AD59" s="11">
-        <v>0.46429999999999999</v>
+        <v>1.1674</v>
       </c>
       <c r="AE59" s="12">
         <v>1</v>
@@ -7790,10 +7790,10 @@
         <v>0</v>
       </c>
       <c r="Y60" s="11">
-        <v>19.03</v>
+        <v>19.690000000000001</v>
       </c>
       <c r="Z60" s="11">
-        <v>19.03</v>
+        <v>19.690000000000001</v>
       </c>
       <c r="AA60" s="12">
         <v>1</v>
@@ -7885,10 +7885,10 @@
         <v>0</v>
       </c>
       <c r="Y61" s="11">
-        <v>58.67</v>
+        <v>61.83</v>
       </c>
       <c r="Z61" s="11">
-        <v>58.67</v>
+        <v>61.83</v>
       </c>
       <c r="AA61" s="12">
         <v>1</v>
@@ -7929,7 +7929,7 @@
         <v>72</v>
       </c>
       <c r="H62" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I62" s="22">
         <v>46000</v>
@@ -8075,10 +8075,10 @@
         <v>0</v>
       </c>
       <c r="Y63" s="11">
-        <v>68.010000000000005</v>
+        <v>70.02</v>
       </c>
       <c r="Z63" s="11">
-        <v>68.010000000000005</v>
+        <v>70.02</v>
       </c>
       <c r="AA63" s="12">
         <v>1</v>
@@ -8134,10 +8134,10 @@
         <v>0</v>
       </c>
       <c r="M64" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N64" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O64" s="12">
         <v>1</v>
@@ -8146,10 +8146,10 @@
         <v>0</v>
       </c>
       <c r="Q64" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R64" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S64" s="12">
         <v>1</v>
@@ -8158,10 +8158,10 @@
         <v>0</v>
       </c>
       <c r="U64" s="11">
-        <v>99.46</v>
+        <v>121.31</v>
       </c>
       <c r="V64" s="11">
-        <v>99.46</v>
+        <v>121.31</v>
       </c>
       <c r="W64" s="12">
         <v>1</v>
@@ -8170,10 +8170,10 @@
         <v>0</v>
       </c>
       <c r="Y64" s="11">
-        <v>20.22</v>
+        <v>25.41</v>
       </c>
       <c r="Z64" s="11">
-        <v>20.22</v>
+        <v>25.41</v>
       </c>
       <c r="AA64" s="12">
         <v>1</v>
@@ -8229,10 +8229,10 @@
         <v>0</v>
       </c>
       <c r="M65" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N65" s="11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O65" s="12">
         <v>1</v>
@@ -8241,22 +8241,22 @@
         <v>0</v>
       </c>
       <c r="Q65" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R65" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S65" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T65" s="11">
         <v>0</v>
       </c>
       <c r="U65" s="11">
-        <v>29.35</v>
+        <v>119.03</v>
       </c>
       <c r="V65" s="11">
-        <v>29.35</v>
+        <v>119.03</v>
       </c>
       <c r="W65" s="12">
         <v>1</v>
@@ -8265,13 +8265,13 @@
         <v>0</v>
       </c>
       <c r="Y65" s="11">
-        <v>0</v>
+        <v>4.99</v>
       </c>
       <c r="Z65" s="11">
-        <v>0</v>
+        <v>4.99</v>
       </c>
       <c r="AA65" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AB65" s="11">
         <v>0</v>
@@ -8294,12 +8294,22 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
+  <conditionalFormatting sqref="A7:A65">
+    <cfRule type="expression" dxfId="68" priority="91" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:A65">
+    <cfRule type="expression" dxfId="67" priority="103" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
     <cfRule type="cellIs" dxfId="61" priority="40" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B65">
+  <conditionalFormatting sqref="B7:B65">
     <cfRule type="expression" dxfId="60" priority="61" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
@@ -8454,7 +8464,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B65">
+  <conditionalFormatting sqref="B7:B65">
     <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
Fix UI crash, precise sheet mapping, and update all campaign data to mid-March
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD5B6BD3-AA51-4149-976E-5C6B39C5D120}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02ABF1C4-BD9E-A846-8D24-F3E21D4C21E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16380" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="2720" yWindow="500" windowWidth="24460" windowHeight="16360" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -665,7 +665,981 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="70">
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="hair">
@@ -856,7 +1830,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="69" headerRowBorderDxfId="68" tableBorderDxfId="67">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -1205,7 +2179,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="1">
-        <v>46092</v>
+        <v>46099</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="46" thickBot="1" x14ac:dyDescent="0.25">
@@ -1281,25 +2255,25 @@
         <v>122</v>
       </c>
       <c r="B5" s="15">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C5" s="15">
-        <v>-77</v>
+        <v>-72</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.63114754098360648</v>
+        <v>-0.5901639344262295</v>
       </c>
       <c r="E5" s="15">
         <v>4684.3999999999996</v>
       </c>
       <c r="F5" s="15">
-        <v>2468.83</v>
+        <v>2670.98</v>
       </c>
       <c r="G5" s="15">
-        <v>-2215.5700000000002</v>
+        <v>-2013.42</v>
       </c>
       <c r="H5" s="16">
-        <v>-0.47296772265391507</v>
+        <v>-0.42981385022628293</v>
       </c>
       <c r="I5" s="15">
         <v>2</v>
@@ -1344,7 +2318,7 @@
   <sheetData>
     <row r="1" spans="1:31" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>46092</v>
+        <v>46099</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1761,13 +2735,13 @@
         <v>5.3364000000000003</v>
       </c>
       <c r="AC7" s="11">
-        <v>6.3615000000000004</v>
+        <v>6.8959000000000001</v>
       </c>
       <c r="AD7" s="11">
-        <v>1.0250999999999999</v>
+        <v>1.5595000000000001</v>
       </c>
       <c r="AE7" s="12">
-        <v>0.19209999999999999</v>
+        <v>0.29220000000000002</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.2">
@@ -1998,13 +2972,13 @@
         <v>1</v>
       </c>
       <c r="M10" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10" s="11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O10" s="12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="P10" s="11">
         <v>1</v>
@@ -2022,13 +2996,13 @@
         <v>29.23</v>
       </c>
       <c r="U10" s="11">
-        <v>0</v>
+        <v>25.2</v>
       </c>
       <c r="V10" s="11">
-        <v>-29.23</v>
+        <v>-4.03</v>
       </c>
       <c r="W10" s="12">
-        <v>-1</v>
+        <v>-0.13789999999999999</v>
       </c>
       <c r="X10" s="11">
         <v>31.17</v>
@@ -2188,13 +3162,13 @@
         <v>8</v>
       </c>
       <c r="M12" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N12" s="11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="O12" s="12">
-        <v>-0.625</v>
+        <v>-0.5</v>
       </c>
       <c r="P12" s="11">
         <v>8</v>
@@ -2212,37 +3186,37 @@
         <v>279.27999999999997</v>
       </c>
       <c r="U12" s="11">
-        <v>75.27</v>
+        <v>179.67</v>
       </c>
       <c r="V12" s="11">
-        <v>-204.01</v>
+        <v>-99.61</v>
       </c>
       <c r="W12" s="12">
-        <v>-0.73050000000000004</v>
+        <v>-0.35670000000000002</v>
       </c>
       <c r="X12" s="11">
         <v>574.09</v>
       </c>
       <c r="Y12" s="11">
-        <v>65.709999999999994</v>
+        <v>73.45</v>
       </c>
       <c r="Z12" s="11">
-        <v>-508.38</v>
+        <v>-500.64</v>
       </c>
       <c r="AA12" s="12">
-        <v>-0.88549999999999995</v>
+        <v>-0.87209999999999999</v>
       </c>
       <c r="AB12" s="11">
         <v>3.1593</v>
       </c>
       <c r="AC12" s="11">
-        <v>17.5944</v>
+        <v>17.987200000000001</v>
       </c>
       <c r="AD12" s="11">
-        <v>14.4351</v>
+        <v>14.8279</v>
       </c>
       <c r="AE12" s="12">
-        <v>4.5690999999999997</v>
+        <v>4.6933999999999996</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
@@ -2331,13 +3305,13 @@
         <v>6.0643000000000002</v>
       </c>
       <c r="AC13" s="11">
-        <v>4.0369999999999999</v>
+        <v>4.2088000000000001</v>
       </c>
       <c r="AD13" s="11">
-        <v>-2.0272999999999999</v>
+        <v>-1.8554999999999999</v>
       </c>
       <c r="AE13" s="12">
-        <v>-0.33429999999999999</v>
+        <v>-0.30599999999999999</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
@@ -2414,13 +3388,13 @@
         <v>27.86</v>
       </c>
       <c r="Y14" s="11">
-        <v>0</v>
+        <v>2.39</v>
       </c>
       <c r="Z14" s="11">
-        <v>-27.86</v>
+        <v>-25.47</v>
       </c>
       <c r="AA14" s="12">
-        <v>-1</v>
+        <v>-0.91420000000000001</v>
       </c>
       <c r="AB14" s="11">
         <v>0</v>
@@ -2458,7 +3432,7 @@
         <v>25</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="I15" s="22">
         <v>43447</v>
@@ -2663,61 +3637,61 @@
         <v>4</v>
       </c>
       <c r="M17" s="11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N17" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O17" s="12">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="P17" s="11">
         <v>6</v>
       </c>
       <c r="Q17" s="11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R17" s="11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S17" s="12">
-        <v>-0.16669999999999999</v>
+        <v>0</v>
       </c>
       <c r="T17" s="11">
         <v>855.64</v>
       </c>
       <c r="U17" s="11">
-        <v>433.01</v>
+        <v>560.76</v>
       </c>
       <c r="V17" s="11">
-        <v>-422.63</v>
+        <v>-294.88</v>
       </c>
       <c r="W17" s="12">
-        <v>-0.49390000000000001</v>
+        <v>-0.34460000000000002</v>
       </c>
       <c r="X17" s="11">
         <v>588.49</v>
       </c>
       <c r="Y17" s="11">
-        <v>633.39</v>
+        <v>699.82</v>
       </c>
       <c r="Z17" s="11">
-        <v>44.9</v>
+        <v>111.33</v>
       </c>
       <c r="AA17" s="12">
-        <v>7.6300000000000007E-2</v>
+        <v>0.18920000000000001</v>
       </c>
       <c r="AB17" s="11">
         <v>0.69879999999999998</v>
       </c>
       <c r="AC17" s="11">
-        <v>0.86550000000000005</v>
+        <v>1.4301999999999999</v>
       </c>
       <c r="AD17" s="11">
-        <v>0.16669999999999999</v>
+        <v>0.73140000000000005</v>
       </c>
       <c r="AE17" s="12">
-        <v>0.23860000000000001</v>
+        <v>1.0467</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.2">
@@ -2889,13 +3863,13 @@
         <v>4.34</v>
       </c>
       <c r="Y19" s="11">
-        <v>10.3</v>
+        <v>15.46</v>
       </c>
       <c r="Z19" s="11">
-        <v>5.96</v>
+        <v>11.12</v>
       </c>
       <c r="AA19" s="12">
-        <v>1.3733</v>
+        <v>2.5621999999999998</v>
       </c>
       <c r="AB19" s="11">
         <v>0</v>
@@ -2972,25 +3946,25 @@
         <v>328.85</v>
       </c>
       <c r="U20" s="11">
-        <v>199.88</v>
+        <v>126.73</v>
       </c>
       <c r="V20" s="11">
-        <v>-128.97</v>
+        <v>-202.12</v>
       </c>
       <c r="W20" s="12">
-        <v>-0.39219999999999999</v>
+        <v>-0.61460000000000004</v>
       </c>
       <c r="X20" s="11">
         <v>353.8</v>
       </c>
       <c r="Y20" s="11">
-        <v>202.83</v>
+        <v>216.24</v>
       </c>
       <c r="Z20" s="11">
-        <v>-150.97</v>
+        <v>-137.56</v>
       </c>
       <c r="AA20" s="12">
-        <v>-0.42670000000000002</v>
+        <v>-0.38879999999999998</v>
       </c>
       <c r="AB20" s="11">
         <v>1.8688</v>
@@ -3091,13 +4065,13 @@
         <v>0.31490000000000001</v>
       </c>
       <c r="AC21" s="11">
-        <v>1.1247</v>
+        <v>1.4286000000000001</v>
       </c>
       <c r="AD21" s="11">
-        <v>0.80979999999999996</v>
+        <v>1.1136999999999999</v>
       </c>
       <c r="AE21" s="12">
-        <v>2.5716000000000001</v>
+        <v>3.5367000000000002</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.2">
@@ -3269,13 +4243,13 @@
         <v>11.9</v>
       </c>
       <c r="Y23" s="11">
-        <v>16.34</v>
+        <v>20.2</v>
       </c>
       <c r="Z23" s="11">
-        <v>4.4400000000000004</v>
+        <v>8.3000000000000007</v>
       </c>
       <c r="AA23" s="12">
-        <v>0.37309999999999999</v>
+        <v>0.69750000000000001</v>
       </c>
       <c r="AB23" s="11">
         <v>0</v>
@@ -3542,25 +4516,25 @@
         <v>58.68</v>
       </c>
       <c r="U26" s="11">
-        <v>24.13</v>
+        <v>-0.1</v>
       </c>
       <c r="V26" s="11">
-        <v>-34.549999999999997</v>
+        <v>-58.78</v>
       </c>
       <c r="W26" s="12">
-        <v>-0.58879999999999999</v>
+        <v>-1.0017</v>
       </c>
       <c r="X26" s="11">
         <v>78.84</v>
       </c>
       <c r="Y26" s="11">
-        <v>46.37</v>
+        <v>48.79</v>
       </c>
       <c r="Z26" s="11">
-        <v>-32.47</v>
+        <v>-30.05</v>
       </c>
       <c r="AA26" s="12">
-        <v>-0.4118</v>
+        <v>-0.38119999999999998</v>
       </c>
       <c r="AB26" s="11">
         <v>0.5141</v>
@@ -3898,61 +4872,61 @@
         <v>8</v>
       </c>
       <c r="M30" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N30" s="11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="O30" s="12">
-        <v>-0.625</v>
+        <v>-0.5</v>
       </c>
       <c r="P30" s="11">
         <v>7</v>
       </c>
       <c r="Q30" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R30" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="S30" s="12">
-        <v>-0.57140000000000002</v>
+        <v>-0.42859999999999998</v>
       </c>
       <c r="T30" s="11">
         <v>224.88</v>
       </c>
       <c r="U30" s="11">
-        <v>86.32</v>
+        <v>112.38</v>
       </c>
       <c r="V30" s="11">
-        <v>-138.56</v>
+        <v>-112.5</v>
       </c>
       <c r="W30" s="12">
-        <v>-0.61619999999999997</v>
+        <v>-0.50029999999999997</v>
       </c>
       <c r="X30" s="11">
         <v>227.28</v>
       </c>
       <c r="Y30" s="11">
-        <v>79.98</v>
+        <v>97.57</v>
       </c>
       <c r="Z30" s="11">
-        <v>-147.30000000000001</v>
+        <v>-129.71</v>
       </c>
       <c r="AA30" s="12">
-        <v>-0.64810000000000001</v>
+        <v>-0.57069999999999999</v>
       </c>
       <c r="AB30" s="11">
         <v>0.1235</v>
       </c>
       <c r="AC30" s="11">
-        <v>0.56420000000000003</v>
+        <v>3.3443000000000001</v>
       </c>
       <c r="AD30" s="11">
-        <v>0.44069999999999998</v>
+        <v>3.2208000000000001</v>
       </c>
       <c r="AE30" s="12">
-        <v>3.5684</v>
+        <v>26.0794</v>
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.2">
@@ -3993,13 +4967,13 @@
         <v>7</v>
       </c>
       <c r="M31" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N31" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="O31" s="12">
-        <v>-0.57140000000000002</v>
+        <v>-0.42859999999999998</v>
       </c>
       <c r="P31" s="11">
         <v>7</v>
@@ -4017,37 +4991,37 @@
         <v>212.51</v>
       </c>
       <c r="U31" s="11">
-        <v>68.92</v>
+        <v>96.98</v>
       </c>
       <c r="V31" s="11">
-        <v>-143.59</v>
+        <v>-115.53</v>
       </c>
       <c r="W31" s="12">
-        <v>-0.67569999999999997</v>
+        <v>-0.54359999999999997</v>
       </c>
       <c r="X31" s="11">
         <v>187.2</v>
       </c>
       <c r="Y31" s="11">
-        <v>58.89</v>
+        <v>56.92</v>
       </c>
       <c r="Z31" s="11">
-        <v>-128.31</v>
+        <v>-130.28</v>
       </c>
       <c r="AA31" s="12">
-        <v>-0.68540000000000001</v>
+        <v>-0.69589999999999996</v>
       </c>
       <c r="AB31" s="11">
         <v>0.79920000000000002</v>
       </c>
       <c r="AC31" s="11">
-        <v>1.1778999999999999</v>
+        <v>1.3084</v>
       </c>
       <c r="AD31" s="11">
-        <v>0.37869999999999998</v>
+        <v>0.50919999999999999</v>
       </c>
       <c r="AE31" s="12">
-        <v>0.4738</v>
+        <v>0.6371</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.2">
@@ -4112,34 +5086,34 @@
         <v>49.3</v>
       </c>
       <c r="U32" s="11">
-        <v>61.31</v>
+        <v>62.71</v>
       </c>
       <c r="V32" s="11">
-        <v>12.01</v>
+        <v>13.41</v>
       </c>
       <c r="W32" s="12">
-        <v>0.24360000000000001</v>
+        <v>0.27200000000000002</v>
       </c>
       <c r="X32" s="11">
         <v>80.510000000000005</v>
       </c>
       <c r="Y32" s="11">
-        <v>26.09</v>
+        <v>30.65</v>
       </c>
       <c r="Z32" s="11">
-        <v>-54.42</v>
+        <v>-49.86</v>
       </c>
       <c r="AA32" s="12">
-        <v>-0.67589999999999995</v>
+        <v>-0.61929999999999996</v>
       </c>
       <c r="AB32" s="11">
         <v>0</v>
       </c>
       <c r="AC32" s="11">
-        <v>0.58040000000000003</v>
+        <v>0.89339999999999997</v>
       </c>
       <c r="AD32" s="11">
-        <v>0.58040000000000003</v>
+        <v>0.89339999999999997</v>
       </c>
       <c r="AE32" s="12">
         <v>1</v>
@@ -4183,49 +5157,49 @@
         <v>2</v>
       </c>
       <c r="M33" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N33" s="11">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="O33" s="12">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="P33" s="11">
         <v>2</v>
       </c>
       <c r="Q33" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R33" s="11">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="S33" s="12">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="T33" s="11">
         <v>67.260000000000005</v>
       </c>
       <c r="U33" s="11">
-        <v>0</v>
+        <v>34.11</v>
       </c>
       <c r="V33" s="11">
-        <v>-67.260000000000005</v>
+        <v>-33.15</v>
       </c>
       <c r="W33" s="12">
-        <v>-1</v>
+        <v>-0.4929</v>
       </c>
       <c r="X33" s="11">
         <v>73</v>
       </c>
       <c r="Y33" s="11">
-        <v>22.78</v>
+        <v>26.42</v>
       </c>
       <c r="Z33" s="11">
-        <v>-50.22</v>
+        <v>-46.58</v>
       </c>
       <c r="AA33" s="12">
-        <v>-0.68789999999999996</v>
+        <v>-0.6381</v>
       </c>
       <c r="AB33" s="11">
         <v>3.1848999999999998</v>
@@ -4314,13 +5288,13 @@
         <v>63.59</v>
       </c>
       <c r="Y34" s="11">
-        <v>72.59</v>
+        <v>98.63</v>
       </c>
       <c r="Z34" s="11">
-        <v>9</v>
+        <v>35.04</v>
       </c>
       <c r="AA34" s="12">
-        <v>0.14149999999999999</v>
+        <v>0.55100000000000005</v>
       </c>
       <c r="AB34" s="11">
         <v>0</v>
@@ -5169,13 +6143,13 @@
         <v>62.03</v>
       </c>
       <c r="Y43" s="11">
-        <v>5.68</v>
+        <v>8.52</v>
       </c>
       <c r="Z43" s="11">
-        <v>-56.35</v>
+        <v>-53.51</v>
       </c>
       <c r="AA43" s="12">
-        <v>-0.90839999999999999</v>
+        <v>-0.86260000000000003</v>
       </c>
       <c r="AB43" s="11">
         <v>0</v>
@@ -5264,13 +6238,13 @@
         <v>44.35</v>
       </c>
       <c r="Y44" s="11">
-        <v>17.68</v>
+        <v>19.739999999999998</v>
       </c>
       <c r="Z44" s="11">
-        <v>-26.67</v>
+        <v>-24.61</v>
       </c>
       <c r="AA44" s="12">
-        <v>-0.60140000000000005</v>
+        <v>-0.55489999999999995</v>
       </c>
       <c r="AB44" s="11">
         <v>0</v>
@@ -5359,25 +6333,25 @@
         <v>156.13999999999999</v>
       </c>
       <c r="Y45" s="11">
-        <v>144.81</v>
+        <v>167.4</v>
       </c>
       <c r="Z45" s="11">
-        <v>-11.33</v>
+        <v>11.26</v>
       </c>
       <c r="AA45" s="12">
-        <v>-7.2599999999999998E-2</v>
+        <v>7.2099999999999997E-2</v>
       </c>
       <c r="AB45" s="11">
         <v>0.2029</v>
       </c>
       <c r="AC45" s="11">
-        <v>0.4355</v>
+        <v>0.4365</v>
       </c>
       <c r="AD45" s="11">
-        <v>0.2326</v>
+        <v>0.2336</v>
       </c>
       <c r="AE45" s="12">
-        <v>1.1464000000000001</v>
+        <v>1.1513</v>
       </c>
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.2">
@@ -6309,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="Y55" s="11">
-        <v>39.47</v>
+        <v>42.53</v>
       </c>
       <c r="Z55" s="11">
-        <v>39.47</v>
+        <v>42.53</v>
       </c>
       <c r="AA55" s="12">
         <v>1</v>
@@ -6368,13 +7342,13 @@
         <v>0</v>
       </c>
       <c r="M56" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N56" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O56" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P56" s="11">
         <v>0</v>
@@ -6392,22 +7366,22 @@
         <v>0</v>
       </c>
       <c r="U56" s="11">
-        <v>0</v>
+        <v>20.22</v>
       </c>
       <c r="V56" s="11">
-        <v>0</v>
+        <v>20.22</v>
       </c>
       <c r="W56" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X56" s="11">
         <v>0</v>
       </c>
       <c r="Y56" s="11">
-        <v>15.97</v>
+        <v>23.77</v>
       </c>
       <c r="Z56" s="11">
-        <v>15.97</v>
+        <v>23.77</v>
       </c>
       <c r="AA56" s="12">
         <v>1</v>
@@ -6879,10 +7853,10 @@
         <v>0</v>
       </c>
       <c r="Y61" s="11">
-        <v>61.83</v>
+        <v>63.6</v>
       </c>
       <c r="Z61" s="11">
-        <v>61.83</v>
+        <v>63.6</v>
       </c>
       <c r="AA61" s="12">
         <v>1</v>
@@ -7113,7 +8087,7 @@
         <v>74</v>
       </c>
       <c r="H64" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="I64" s="22">
         <v>46007</v>
@@ -7140,10 +8114,10 @@
         <v>0</v>
       </c>
       <c r="Q64" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R64" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S64" s="12">
         <v>1</v>
@@ -7164,10 +8138,10 @@
         <v>0</v>
       </c>
       <c r="Y64" s="11">
-        <v>25.41</v>
+        <v>31.24</v>
       </c>
       <c r="Z64" s="11">
-        <v>25.41</v>
+        <v>31.24</v>
       </c>
       <c r="AA64" s="12">
         <v>1</v>
@@ -7235,10 +8209,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R65" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S65" s="12">
         <v>1</v>
@@ -7259,10 +8233,10 @@
         <v>0</v>
       </c>
       <c r="Y65" s="11">
-        <v>4.99</v>
+        <v>9.92</v>
       </c>
       <c r="Z65" s="11">
-        <v>4.99</v>
+        <v>9.92</v>
       </c>
       <c r="AA65" s="12">
         <v>1</v>
@@ -7288,37 +8262,312 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A7:W65">
-    <cfRule type="expression" dxfId="6" priority="41" stopIfTrue="1">
+  <conditionalFormatting sqref="A7:B65">
+    <cfRule type="expression" dxfId="66" priority="101" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:C65">
-    <cfRule type="expression" dxfId="5" priority="29" stopIfTrue="1">
+  <conditionalFormatting sqref="B7:B65">
+    <cfRule type="expression" dxfId="65" priority="89" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D7:V65">
-    <cfRule type="expression" dxfId="4" priority="10">
+  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
+    <cfRule type="cellIs" dxfId="59" priority="39" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7:C65">
+    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N7:O65 R7:S65 V7:W65 Z7:AA65 AD7:AE65">
-    <cfRule type="cellIs" dxfId="3" priority="9" operator="lessThan">
+  <conditionalFormatting sqref="D7:D65">
+    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7:E65">
+    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F65">
+    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:G65">
+    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H65">
+    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:I65">
+    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:J65">
+    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K65">
+    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:L65">
+    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7:M65">
+    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N65">
+    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O7:O65">
+    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:P65">
+    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q7:Q65">
+    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R65">
+    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S7:S65">
+    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T7:T65">
+    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:U65">
+    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V7:V65">
+    <cfRule type="expression" dxfId="39" priority="40" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:W65">
+    <cfRule type="expression" dxfId="38" priority="60" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X7:X65">
+    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Y65">
+    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z7:Z65">
+    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA7:AA65">
+    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB7:AB65">
+    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC7:AC65">
+    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD65">
+    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE7:AE65">
+    <cfRule type="expression" dxfId="30" priority="31" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
+    <cfRule type="cellIs" dxfId="29" priority="9" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V7:W65 Z7:AA65 AD7:AE65 N7:O65 R7:S65">
-    <cfRule type="cellIs" dxfId="2" priority="40" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:AE65">
-    <cfRule type="expression" dxfId="1" priority="31" stopIfTrue="1">
+  <conditionalFormatting sqref="C7:C65">
+    <cfRule type="expression" dxfId="28" priority="29" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X7:AE65">
+  <conditionalFormatting sqref="D7:D65">
+    <cfRule type="expression" dxfId="27" priority="28">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7:E65">
+    <cfRule type="expression" dxfId="26" priority="27">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F65">
+    <cfRule type="expression" dxfId="25" priority="26">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:G65">
+    <cfRule type="expression" dxfId="24" priority="25">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H65">
+    <cfRule type="expression" dxfId="23" priority="24">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:I65">
+    <cfRule type="expression" dxfId="22" priority="23">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:J65">
+    <cfRule type="expression" dxfId="21" priority="22">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K65">
+    <cfRule type="expression" dxfId="20" priority="21">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:L65">
+    <cfRule type="expression" dxfId="19" priority="20">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7:M65">
+    <cfRule type="expression" dxfId="18" priority="19">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N65">
+    <cfRule type="expression" dxfId="17" priority="18">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O7:O65">
+    <cfRule type="expression" dxfId="16" priority="17">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:P65">
+    <cfRule type="expression" dxfId="15" priority="16">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q7:Q65">
+    <cfRule type="expression" dxfId="14" priority="15">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R65">
+    <cfRule type="expression" dxfId="13" priority="14">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S7:S65">
+    <cfRule type="expression" dxfId="12" priority="13">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T7:T65">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:U65">
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V7:V65">
+    <cfRule type="expression" dxfId="9" priority="10">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:W65">
+    <cfRule type="expression" dxfId="8" priority="30" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X7:X65">
+    <cfRule type="expression" dxfId="7" priority="8">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Y65">
+    <cfRule type="expression" dxfId="6" priority="7">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z7:Z65">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA7:AA65">
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB7:AB65">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC7:AC65">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD65">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE7:AE65">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: push updated report snapshot (March 26)
- Included the newly generated 'resumen_snapshot.json' in the repo
  to ensure the production site reflects the latest campaign and
  admin report data instantly.
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02ABF1C4-BD9E-A846-8D24-F3E21D4C21E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB99C0D9-F878-1842-BB47-DE1D0141D6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2720" yWindow="500" windowWidth="24460" windowHeight="16360" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -665,7 +665,23 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="70">
+  <dxfs count="72">
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="hair">
@@ -1138,6 +1154,22 @@
         <extend val="0"/>
         <color indexed="10"/>
       </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -1830,7 +1862,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="69" headerRowBorderDxfId="68" tableBorderDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="71" headerRowBorderDxfId="70" tableBorderDxfId="69">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -2179,7 +2211,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="1">
-        <v>46099</v>
+        <v>46101</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="46" thickBot="1" x14ac:dyDescent="0.25">
@@ -2255,25 +2287,25 @@
         <v>122</v>
       </c>
       <c r="B5" s="15">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C5" s="15">
-        <v>-72</v>
+        <v>-66</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.5901639344262295</v>
+        <v>-0.54098360655737698</v>
       </c>
       <c r="E5" s="15">
         <v>4684.3999999999996</v>
       </c>
       <c r="F5" s="15">
-        <v>2670.98</v>
+        <v>2927.66</v>
       </c>
       <c r="G5" s="15">
-        <v>-2013.42</v>
+        <v>-1756.74</v>
       </c>
       <c r="H5" s="16">
-        <v>-0.42981385022628293</v>
+        <v>-0.37501921270600291</v>
       </c>
       <c r="I5" s="15">
         <v>2</v>
@@ -2318,7 +2350,7 @@
   <sheetData>
     <row r="1" spans="1:31" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>46099</v>
+        <v>46101</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -2494,64 +2526,64 @@
       <c r="J5" s="19"/>
       <c r="K5" s="19"/>
       <c r="L5" s="15">
-        <v>87</v>
+        <v>127</v>
       </c>
       <c r="M5" s="15">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="N5" s="15">
-        <v>-43</v>
+        <v>-63</v>
       </c>
       <c r="O5" s="16">
-        <v>-0.49425287356321834</v>
+        <v>-0.49606299212598426</v>
       </c>
       <c r="P5" s="15">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="Q5" s="15">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="R5" s="15">
-        <v>-40</v>
+        <v>-66</v>
       </c>
       <c r="S5" s="16">
-        <v>-0.51282051282051277</v>
+        <v>-0.54098360655737698</v>
       </c>
       <c r="T5" s="15">
-        <v>3345.28</v>
+        <v>4754.3900000000003</v>
       </c>
       <c r="U5" s="15">
-        <v>162.23999999999981</v>
+        <v>1112.4400000000003</v>
       </c>
       <c r="V5" s="15">
-        <v>-3183.0400000000004</v>
+        <v>-3641.9499999999994</v>
       </c>
       <c r="W5" s="16">
-        <v>-0.95150181748612972</v>
+        <v>-0.76601835356375891</v>
       </c>
       <c r="X5" s="15">
-        <v>3065.0899999999988</v>
+        <v>4684.4000000000005</v>
       </c>
       <c r="Y5" s="15">
-        <v>1888.5900000000001</v>
+        <v>2927.6599999999994</v>
       </c>
       <c r="Z5" s="15">
-        <v>-1176.5000000000002</v>
+        <v>-1756.7399999999998</v>
       </c>
       <c r="AA5" s="16">
-        <v>-0.38383864747854035</v>
+        <v>-0.37501921270600314</v>
       </c>
       <c r="AB5" s="15">
-        <v>21.1402</v>
+        <v>29.353999999999996</v>
       </c>
       <c r="AC5" s="15">
-        <v>31.525700000000001</v>
+        <v>57.281699999999994</v>
       </c>
       <c r="AD5" s="15">
-        <v>10.3855</v>
+        <v>27.927700000000005</v>
       </c>
       <c r="AE5" s="16">
-        <v>0.4912678214964854</v>
+        <v>0.95141036996661454</v>
       </c>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.2">
@@ -3162,49 +3194,49 @@
         <v>8</v>
       </c>
       <c r="M12" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N12" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="O12" s="12">
-        <v>-0.5</v>
+        <v>-0.375</v>
       </c>
       <c r="P12" s="11">
         <v>8</v>
       </c>
       <c r="Q12" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R12" s="11">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="S12" s="12">
-        <v>-0.625</v>
+        <v>-0.5</v>
       </c>
       <c r="T12" s="11">
         <v>279.27999999999997</v>
       </c>
       <c r="U12" s="11">
-        <v>179.67</v>
+        <v>205.06</v>
       </c>
       <c r="V12" s="11">
-        <v>-99.61</v>
+        <v>-74.22</v>
       </c>
       <c r="W12" s="12">
-        <v>-0.35670000000000002</v>
+        <v>-0.26579999999999998</v>
       </c>
       <c r="X12" s="11">
         <v>574.09</v>
       </c>
       <c r="Y12" s="11">
-        <v>73.45</v>
+        <v>170.7</v>
       </c>
       <c r="Z12" s="11">
-        <v>-500.64</v>
+        <v>-403.39</v>
       </c>
       <c r="AA12" s="12">
-        <v>-0.87209999999999999</v>
+        <v>-0.70269999999999999</v>
       </c>
       <c r="AB12" s="11">
         <v>3.1593</v>
@@ -3673,13 +3705,13 @@
         <v>588.49</v>
       </c>
       <c r="Y17" s="11">
-        <v>699.82</v>
+        <v>702.8</v>
       </c>
       <c r="Z17" s="11">
-        <v>111.33</v>
+        <v>114.31</v>
       </c>
       <c r="AA17" s="12">
-        <v>0.18920000000000001</v>
+        <v>0.19420000000000001</v>
       </c>
       <c r="AB17" s="11">
         <v>0.69879999999999998</v>
@@ -4017,10 +4049,10 @@
         <v>0</v>
       </c>
       <c r="M21" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N21" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O21" s="12">
         <v>1</v>
@@ -4041,10 +4073,10 @@
         <v>0</v>
       </c>
       <c r="U21" s="11">
-        <v>111.57</v>
+        <v>139</v>
       </c>
       <c r="V21" s="11">
-        <v>111.57</v>
+        <v>139</v>
       </c>
       <c r="W21" s="12">
         <v>1</v>
@@ -4908,13 +4940,13 @@
         <v>227.28</v>
       </c>
       <c r="Y30" s="11">
-        <v>97.57</v>
+        <v>99.18</v>
       </c>
       <c r="Z30" s="11">
-        <v>-129.71</v>
+        <v>-128.1</v>
       </c>
       <c r="AA30" s="12">
-        <v>-0.57069999999999999</v>
+        <v>-0.56359999999999999</v>
       </c>
       <c r="AB30" s="11">
         <v>0.1235</v>
@@ -4967,61 +4999,61 @@
         <v>7</v>
       </c>
       <c r="M31" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N31" s="11">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="O31" s="12">
-        <v>-0.42859999999999998</v>
+        <v>-0.28570000000000001</v>
       </c>
       <c r="P31" s="11">
         <v>7</v>
       </c>
       <c r="Q31" s="11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R31" s="11">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="S31" s="12">
-        <v>-0.57140000000000002</v>
+        <v>-0.28570000000000001</v>
       </c>
       <c r="T31" s="11">
         <v>212.51</v>
       </c>
       <c r="U31" s="11">
-        <v>96.98</v>
+        <v>132.76</v>
       </c>
       <c r="V31" s="11">
-        <v>-115.53</v>
+        <v>-79.75</v>
       </c>
       <c r="W31" s="12">
-        <v>-0.54359999999999997</v>
+        <v>-0.37530000000000002</v>
       </c>
       <c r="X31" s="11">
         <v>187.2</v>
       </c>
       <c r="Y31" s="11">
-        <v>56.92</v>
+        <v>122.51</v>
       </c>
       <c r="Z31" s="11">
-        <v>-130.28</v>
+        <v>-64.69</v>
       </c>
       <c r="AA31" s="12">
-        <v>-0.69589999999999996</v>
+        <v>-0.34560000000000002</v>
       </c>
       <c r="AB31" s="11">
         <v>0.79920000000000002</v>
       </c>
       <c r="AC31" s="11">
-        <v>1.3084</v>
+        <v>1.4389000000000001</v>
       </c>
       <c r="AD31" s="11">
-        <v>0.50919999999999999</v>
+        <v>0.63970000000000005</v>
       </c>
       <c r="AE31" s="12">
-        <v>0.6371</v>
+        <v>0.8004</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.2">
@@ -5074,13 +5106,13 @@
         <v>2</v>
       </c>
       <c r="Q32" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R32" s="11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S32" s="12">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="T32" s="11">
         <v>49.3</v>
@@ -5098,13 +5130,13 @@
         <v>80.510000000000005</v>
       </c>
       <c r="Y32" s="11">
-        <v>30.65</v>
+        <v>65.56</v>
       </c>
       <c r="Z32" s="11">
-        <v>-49.86</v>
+        <v>-14.95</v>
       </c>
       <c r="AA32" s="12">
-        <v>-0.61929999999999996</v>
+        <v>-0.1857</v>
       </c>
       <c r="AB32" s="11">
         <v>0</v>
@@ -5193,13 +5225,13 @@
         <v>73</v>
       </c>
       <c r="Y33" s="11">
-        <v>26.42</v>
+        <v>28.89</v>
       </c>
       <c r="Z33" s="11">
-        <v>-46.58</v>
+        <v>-44.11</v>
       </c>
       <c r="AA33" s="12">
-        <v>-0.6381</v>
+        <v>-0.60419999999999996</v>
       </c>
       <c r="AB33" s="11">
         <v>3.1848999999999998</v>
@@ -5288,13 +5320,13 @@
         <v>63.59</v>
       </c>
       <c r="Y34" s="11">
-        <v>98.63</v>
+        <v>104.69</v>
       </c>
       <c r="Z34" s="11">
-        <v>35.04</v>
+        <v>41.1</v>
       </c>
       <c r="AA34" s="12">
-        <v>0.55100000000000005</v>
+        <v>0.64629999999999999</v>
       </c>
       <c r="AB34" s="11">
         <v>0</v>
@@ -5490,13 +5522,13 @@
         <v>4.0427</v>
       </c>
       <c r="AC36" s="11">
-        <v>2.7980999999999998</v>
+        <v>7.7786</v>
       </c>
       <c r="AD36" s="11">
-        <v>-1.2445999999999999</v>
+        <v>3.7359</v>
       </c>
       <c r="AE36" s="12">
-        <v>-0.30790000000000001</v>
+        <v>0.92410000000000003</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.2">
@@ -5858,13 +5890,13 @@
         <v>29.29</v>
       </c>
       <c r="Y40" s="11">
-        <v>16.809999999999999</v>
+        <v>18.170000000000002</v>
       </c>
       <c r="Z40" s="11">
-        <v>-12.48</v>
+        <v>-11.12</v>
       </c>
       <c r="AA40" s="12">
-        <v>-0.42609999999999998</v>
+        <v>-0.37969999999999998</v>
       </c>
       <c r="AB40" s="11">
         <v>0</v>
@@ -6238,13 +6270,13 @@
         <v>44.35</v>
       </c>
       <c r="Y44" s="11">
-        <v>19.739999999999998</v>
+        <v>26.54</v>
       </c>
       <c r="Z44" s="11">
-        <v>-24.61</v>
+        <v>-17.809999999999999</v>
       </c>
       <c r="AA44" s="12">
-        <v>-0.55489999999999995</v>
+        <v>-0.40160000000000001</v>
       </c>
       <c r="AB44" s="11">
         <v>0</v>
@@ -6998,13 +7030,13 @@
         <v>2.4500000000000002</v>
       </c>
       <c r="Y52" s="11">
-        <v>13.31</v>
+        <v>15.04</v>
       </c>
       <c r="Z52" s="11">
-        <v>10.86</v>
+        <v>12.59</v>
       </c>
       <c r="AA52" s="12">
-        <v>4.4326999999999996</v>
+        <v>5.1387999999999998</v>
       </c>
       <c r="AB52" s="11">
         <v>0</v>
@@ -7188,10 +7220,10 @@
         <v>0</v>
       </c>
       <c r="Y54" s="11">
-        <v>67.709999999999994</v>
+        <v>69.489999999999995</v>
       </c>
       <c r="Z54" s="11">
-        <v>67.709999999999994</v>
+        <v>69.489999999999995</v>
       </c>
       <c r="AA54" s="12">
         <v>1</v>
@@ -7283,10 +7315,10 @@
         <v>0</v>
       </c>
       <c r="Y55" s="11">
-        <v>42.53</v>
+        <v>45.5</v>
       </c>
       <c r="Z55" s="11">
-        <v>42.53</v>
+        <v>45.5</v>
       </c>
       <c r="AA55" s="12">
         <v>1</v>
@@ -7354,13 +7386,13 @@
         <v>0</v>
       </c>
       <c r="Q56" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R56" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S56" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T56" s="11">
         <v>0</v>
@@ -7378,10 +7410,10 @@
         <v>0</v>
       </c>
       <c r="Y56" s="11">
-        <v>23.77</v>
+        <v>25.46</v>
       </c>
       <c r="Z56" s="11">
-        <v>23.77</v>
+        <v>25.46</v>
       </c>
       <c r="AA56" s="12">
         <v>1</v>
@@ -7473,10 +7505,10 @@
         <v>0</v>
       </c>
       <c r="Y57" s="11">
-        <v>18.93</v>
+        <v>20.6</v>
       </c>
       <c r="Z57" s="11">
-        <v>18.93</v>
+        <v>20.6</v>
       </c>
       <c r="AA57" s="12">
         <v>1</v>
@@ -7639,10 +7671,10 @@
         <v>0</v>
       </c>
       <c r="Q59" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R59" s="11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S59" s="12">
         <v>1</v>
@@ -7663,10 +7695,10 @@
         <v>0</v>
       </c>
       <c r="Y59" s="11">
-        <v>110.56</v>
+        <v>136.78</v>
       </c>
       <c r="Z59" s="11">
-        <v>110.56</v>
+        <v>136.78</v>
       </c>
       <c r="AA59" s="12">
         <v>1</v>
@@ -7948,10 +7980,10 @@
         <v>0</v>
       </c>
       <c r="Y62" s="11">
-        <v>3.16</v>
+        <v>4.75</v>
       </c>
       <c r="Z62" s="11">
-        <v>3.16</v>
+        <v>4.75</v>
       </c>
       <c r="AA62" s="12">
         <v>1</v>
@@ -8087,7 +8119,7 @@
         <v>74</v>
       </c>
       <c r="H64" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I64" s="22">
         <v>46007</v>
@@ -8262,169 +8294,169 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
+  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
+    <cfRule type="cellIs" dxfId="61" priority="40" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A7:B65">
-    <cfRule type="expression" dxfId="66" priority="101" stopIfTrue="1">
+    <cfRule type="expression" dxfId="60" priority="61" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B7:B65">
-    <cfRule type="expression" dxfId="65" priority="89" stopIfTrue="1">
+  <conditionalFormatting sqref="C7:C65">
+    <cfRule type="expression" dxfId="59" priority="60" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:D65">
+    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7:E65">
+    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F65">
+    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:G65">
+    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H65">
+    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:I65">
+    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:J65">
+    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K65">
+    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:L65">
+    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7:M65">
+    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N65">
+    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O7:O65">
+    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:P65">
+    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q7:Q65">
+    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R65">
+    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S7:S65">
+    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T7:T65">
+    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:U65">
+    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V7:V65">
+    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:W65">
+    <cfRule type="expression" dxfId="39" priority="62" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X7:X65">
+    <cfRule type="expression" dxfId="38" priority="39" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Y65">
+    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z7:Z65">
+    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA7:AA65">
+    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB7:AB65">
+    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC7:AC65">
+    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD65">
+    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE7:AE65">
+    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
-    <cfRule type="cellIs" dxfId="59" priority="39" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="30" priority="9" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C7:C65">
-    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
+  <conditionalFormatting sqref="A7:B65">
+    <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D65">
-    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E65">
-    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F65">
-    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G65">
-    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H65">
-    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I65">
-    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J65">
-    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K65">
-    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L65">
-    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M65">
-    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N65">
-    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O7:O65">
-    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P65">
-    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q7:Q65">
-    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R7:R65">
-    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S65">
-    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T7:T65">
-    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U65">
-    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7:V65">
-    <cfRule type="expression" dxfId="39" priority="40" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:W65">
-    <cfRule type="expression" dxfId="38" priority="60" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X7:X65">
-    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Y65">
-    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z7:Z65">
-    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA65">
-    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB7:AB65">
-    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7:AC65">
-    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AD65">
-    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE7:AE65">
-    <cfRule type="expression" dxfId="30" priority="31" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
-    <cfRule type="cellIs" dxfId="29" priority="9" operator="lessThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C65">
@@ -8528,7 +8560,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W7:W65">
-    <cfRule type="expression" dxfId="8" priority="30" stopIfTrue="1">
+    <cfRule type="expression" dxfId="8" priority="31" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
update: refresh campaign reports and snapshot for March 31 cierre
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB99C0D9-F878-1842-BB47-DE1D0141D6D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76F1B9D-9BAB-5F4A-B99D-8F494D9AD651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -665,1013 +665,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="72">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <border>
         <left style="hair">
@@ -1862,7 +856,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="71" headerRowBorderDxfId="70" tableBorderDxfId="69">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -8294,312 +7288,37 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
-  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
-    <cfRule type="cellIs" dxfId="61" priority="40" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="A7:C65">
+    <cfRule type="expression" dxfId="6" priority="29" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:W65">
+    <cfRule type="expression" dxfId="5" priority="41" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:V65">
+    <cfRule type="expression" dxfId="4" priority="10">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:O65 R7:S65 V7:W65 Z7:AA65 AD7:AE65">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B65">
-    <cfRule type="expression" dxfId="60" priority="61" stopIfTrue="1">
+  <conditionalFormatting sqref="V7:W65 Z7:AA65 AD7:AE65 N7:O65 R7:S65">
+    <cfRule type="cellIs" dxfId="2" priority="40" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:AE65">
+    <cfRule type="expression" dxfId="1" priority="31" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C7:C65">
-    <cfRule type="expression" dxfId="59" priority="60" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D65">
-    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E65">
-    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F65">
-    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G65">
-    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H65">
-    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I65">
-    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J65">
-    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K65">
-    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L65">
-    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M65">
-    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N65">
-    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O7:O65">
-    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P65">
-    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q7:Q65">
-    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R7:R65">
-    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S65">
-    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T7:T65">
-    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U65">
-    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7:V65">
-    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:W65">
-    <cfRule type="expression" dxfId="39" priority="62" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X7:X65">
-    <cfRule type="expression" dxfId="38" priority="39" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Y65">
-    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z7:Z65">
-    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA65">
-    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB7:AB65">
-    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7:AC65">
-    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AD65">
-    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE7:AE65">
-    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AE65 N7:O65 R7:S65 V7:W65 Z7:AA65">
-    <cfRule type="cellIs" dxfId="30" priority="9" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B65">
-    <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7:C65">
-    <cfRule type="expression" dxfId="28" priority="29" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D65">
-    <cfRule type="expression" dxfId="27" priority="28">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E65">
-    <cfRule type="expression" dxfId="26" priority="27">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F65">
-    <cfRule type="expression" dxfId="25" priority="26">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G65">
-    <cfRule type="expression" dxfId="24" priority="25">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H65">
-    <cfRule type="expression" dxfId="23" priority="24">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I65">
-    <cfRule type="expression" dxfId="22" priority="23">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J65">
-    <cfRule type="expression" dxfId="21" priority="22">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K65">
-    <cfRule type="expression" dxfId="20" priority="21">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L65">
-    <cfRule type="expression" dxfId="19" priority="20">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M65">
-    <cfRule type="expression" dxfId="18" priority="19">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N65">
-    <cfRule type="expression" dxfId="17" priority="18">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O7:O65">
-    <cfRule type="expression" dxfId="16" priority="17">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P65">
-    <cfRule type="expression" dxfId="15" priority="16">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q7:Q65">
-    <cfRule type="expression" dxfId="14" priority="15">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R7:R65">
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S65">
-    <cfRule type="expression" dxfId="12" priority="13">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T7:T65">
-    <cfRule type="expression" dxfId="11" priority="12">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U65">
-    <cfRule type="expression" dxfId="10" priority="11">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7:V65">
-    <cfRule type="expression" dxfId="9" priority="10">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:W65">
-    <cfRule type="expression" dxfId="8" priority="31" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X7:X65">
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Y65">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z7:Z65">
-    <cfRule type="expression" dxfId="5" priority="6">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA65">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB7:AB65">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7:AC65">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AD65">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE7:AE65">
+  <conditionalFormatting sqref="X7:AE65">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
Actualización de campañas y resumen de asesores al 31 de marzo
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76F1B9D-9BAB-5F4A-B99D-8F494D9AD651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8E8360-929D-C74A-BB41-15CF60D3ADB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="100" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="136">
   <si>
     <t>Asesor</t>
   </si>
@@ -439,6 +439,12 @@
   </si>
   <si>
     <t>MONSERRAT VELASCO SANTOS</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>MARIO IVAN ROMERO GONZALEZ</t>
   </si>
 </sst>
 </file>
@@ -449,7 +455,7 @@
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -495,6 +501,12 @@
     <font>
       <sz val="10"/>
       <color indexed="9"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -665,7 +677,455 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="136">
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <border>
         <left style="hair">
@@ -722,6 +1182,486 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -793,17 +1733,1007 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="double">
+          <color indexed="22"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="double">
           <color indexed="22"/>
         </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="double">
-          <color indexed="22"/>
-        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -842,6 +2772,132 @@
       </border>
       <protection locked="1" hidden="1"/>
     </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -856,7 +2912,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="128" headerRowBorderDxfId="126" tableBorderDxfId="127">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -1205,7 +3261,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="1">
-        <v>46101</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="46" thickBot="1" x14ac:dyDescent="0.25">
@@ -1281,52 +3337,53 @@
         <v>122</v>
       </c>
       <c r="B5" s="15">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="C5" s="15">
-        <v>-66</v>
+        <v>-56</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.54098360655737698</v>
+        <v>-0.45901639344262291</v>
       </c>
       <c r="E5" s="15">
         <v>4684.3999999999996</v>
       </c>
       <c r="F5" s="15">
-        <v>2927.66</v>
+        <v>3371.71</v>
       </c>
       <c r="G5" s="15">
-        <v>-1756.74</v>
+        <v>-1312.69</v>
       </c>
       <c r="H5" s="16">
-        <v>-0.37501921270600291</v>
+        <v>-0.2802258560327896</v>
       </c>
       <c r="I5" s="15">
         <v>2</v>
       </c>
       <c r="J5" s="15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="15">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="L5" s="16">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="M5" s="15">
         <v>313.24</v>
       </c>
       <c r="N5" s="15">
-        <v>0</v>
+        <v>72.052099999999996</v>
       </c>
       <c r="O5" s="15">
-        <v>-313.24</v>
+        <v>-241.18790000000001</v>
       </c>
       <c r="P5" s="16">
-        <v>-1</v>
+        <v>-0.76997797216192065</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -1336,7 +3393,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6395312-445F-3747-AD98-F1F037E33F44}">
-  <dimension ref="A1:AE65"/>
+  <dimension ref="A1:AE66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" bestFit="1" customWidth="1"/>
@@ -1344,7 +3401,7 @@
   <sheetData>
     <row r="1" spans="1:31" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>46101</v>
+        <v>46112</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1713,61 +3770,61 @@
         <v>4</v>
       </c>
       <c r="M7" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N7" s="11">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="O7" s="12">
-        <v>-0.5</v>
+        <v>0</v>
       </c>
       <c r="P7" s="11">
         <v>4</v>
       </c>
       <c r="Q7" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R7" s="11">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="S7" s="12">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="T7" s="11">
         <v>134.32</v>
       </c>
       <c r="U7" s="11">
-        <v>61.9</v>
+        <v>134.38999999999999</v>
       </c>
       <c r="V7" s="11">
-        <v>-72.42</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="W7" s="12">
-        <v>-0.53920000000000001</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="X7" s="11">
         <v>238.93</v>
       </c>
       <c r="Y7" s="11">
-        <v>115.62</v>
+        <v>178.07</v>
       </c>
       <c r="Z7" s="11">
-        <v>-123.31</v>
+        <v>-60.86</v>
       </c>
       <c r="AA7" s="12">
-        <v>-0.5161</v>
+        <v>-0.25469999999999998</v>
       </c>
       <c r="AB7" s="11">
         <v>5.3364000000000003</v>
       </c>
       <c r="AC7" s="11">
-        <v>6.8959000000000001</v>
+        <v>8.8035999999999994</v>
       </c>
       <c r="AD7" s="11">
-        <v>1.5595000000000001</v>
+        <v>3.4672000000000001</v>
       </c>
       <c r="AE7" s="12">
-        <v>0.29220000000000002</v>
+        <v>0.64970000000000006</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.2">
@@ -1939,13 +3996,13 @@
         <v>31.29</v>
       </c>
       <c r="Y9" s="11">
-        <v>7.18</v>
+        <v>9.02</v>
       </c>
       <c r="Z9" s="11">
-        <v>-24.11</v>
+        <v>-22.27</v>
       </c>
       <c r="AA9" s="12">
-        <v>-0.77049999999999996</v>
+        <v>-0.7117</v>
       </c>
       <c r="AB9" s="11">
         <v>0</v>
@@ -2010,37 +4067,37 @@
         <v>1</v>
       </c>
       <c r="Q10" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R10" s="11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T10" s="11">
         <v>29.23</v>
       </c>
       <c r="U10" s="11">
-        <v>25.2</v>
+        <v>25.39</v>
       </c>
       <c r="V10" s="11">
-        <v>-4.03</v>
+        <v>-3.84</v>
       </c>
       <c r="W10" s="12">
-        <v>-0.13789999999999999</v>
+        <v>-0.13139999999999999</v>
       </c>
       <c r="X10" s="11">
         <v>31.17</v>
       </c>
       <c r="Y10" s="11">
-        <v>5.51</v>
+        <v>33.700000000000003</v>
       </c>
       <c r="Z10" s="11">
-        <v>-25.66</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="AA10" s="12">
-        <v>-0.82320000000000004</v>
+        <v>8.1199999999999994E-2</v>
       </c>
       <c r="AB10" s="11">
         <v>0</v>
@@ -2188,61 +4245,61 @@
         <v>8</v>
       </c>
       <c r="M12" s="11">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N12" s="11">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="O12" s="12">
-        <v>-0.375</v>
+        <v>0</v>
       </c>
       <c r="P12" s="11">
         <v>8</v>
       </c>
       <c r="Q12" s="11">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R12" s="11">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="S12" s="12">
-        <v>-0.5</v>
+        <v>-0.25</v>
       </c>
       <c r="T12" s="11">
         <v>279.27999999999997</v>
       </c>
       <c r="U12" s="11">
-        <v>205.06</v>
+        <v>357.98</v>
       </c>
       <c r="V12" s="11">
-        <v>-74.22</v>
+        <v>78.7</v>
       </c>
       <c r="W12" s="12">
-        <v>-0.26579999999999998</v>
+        <v>0.28179999999999999</v>
       </c>
       <c r="X12" s="11">
         <v>574.09</v>
       </c>
       <c r="Y12" s="11">
-        <v>170.7</v>
+        <v>249.15</v>
       </c>
       <c r="Z12" s="11">
-        <v>-403.39</v>
+        <v>-324.94</v>
       </c>
       <c r="AA12" s="12">
-        <v>-0.70269999999999999</v>
+        <v>-0.56599999999999995</v>
       </c>
       <c r="AB12" s="11">
         <v>3.1593</v>
       </c>
       <c r="AC12" s="11">
-        <v>17.987200000000001</v>
+        <v>19.947700000000001</v>
       </c>
       <c r="AD12" s="11">
-        <v>14.8279</v>
+        <v>16.788399999999999</v>
       </c>
       <c r="AE12" s="12">
-        <v>4.6933999999999996</v>
+        <v>5.3140000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
@@ -2319,25 +4376,25 @@
         <v>99.88</v>
       </c>
       <c r="Y13" s="11">
-        <v>30.24</v>
+        <v>39.76</v>
       </c>
       <c r="Z13" s="11">
-        <v>-69.64</v>
+        <v>-60.12</v>
       </c>
       <c r="AA13" s="12">
-        <v>-0.69720000000000004</v>
+        <v>-0.60189999999999999</v>
       </c>
       <c r="AB13" s="11">
         <v>6.0643000000000002</v>
       </c>
       <c r="AC13" s="11">
-        <v>4.2088000000000001</v>
+        <v>6.2045000000000003</v>
       </c>
       <c r="AD13" s="11">
-        <v>-1.8554999999999999</v>
+        <v>0.14019999999999999</v>
       </c>
       <c r="AE13" s="12">
-        <v>-0.30599999999999999</v>
+        <v>2.3099999999999999E-2</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
@@ -2414,13 +4471,13 @@
         <v>27.86</v>
       </c>
       <c r="Y14" s="11">
-        <v>2.39</v>
+        <v>2.4</v>
       </c>
       <c r="Z14" s="11">
-        <v>-25.47</v>
+        <v>-25.46</v>
       </c>
       <c r="AA14" s="12">
-        <v>-0.91420000000000001</v>
+        <v>-0.91390000000000005</v>
       </c>
       <c r="AB14" s="11">
         <v>0</v>
@@ -2521,10 +4578,10 @@
         <v>0</v>
       </c>
       <c r="AC15" s="11">
-        <v>3.2017000000000002</v>
+        <v>6.7150999999999996</v>
       </c>
       <c r="AD15" s="11">
-        <v>3.2017000000000002</v>
+        <v>6.7150999999999996</v>
       </c>
       <c r="AE15" s="12">
         <v>1</v>
@@ -2663,61 +4720,61 @@
         <v>4</v>
       </c>
       <c r="M17" s="11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N17" s="11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="O17" s="12">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="P17" s="11">
         <v>6</v>
       </c>
       <c r="Q17" s="11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R17" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="12">
-        <v>0</v>
+        <v>0.16669999999999999</v>
       </c>
       <c r="T17" s="11">
         <v>855.64</v>
       </c>
       <c r="U17" s="11">
-        <v>560.76</v>
+        <v>670.28</v>
       </c>
       <c r="V17" s="11">
-        <v>-294.88</v>
+        <v>-185.36</v>
       </c>
       <c r="W17" s="12">
-        <v>-0.34460000000000002</v>
+        <v>-0.21659999999999999</v>
       </c>
       <c r="X17" s="11">
         <v>588.49</v>
       </c>
       <c r="Y17" s="11">
-        <v>702.8</v>
+        <v>760.86</v>
       </c>
       <c r="Z17" s="11">
-        <v>114.31</v>
+        <v>172.37</v>
       </c>
       <c r="AA17" s="12">
-        <v>0.19420000000000001</v>
+        <v>0.29289999999999999</v>
       </c>
       <c r="AB17" s="11">
         <v>0.69879999999999998</v>
       </c>
       <c r="AC17" s="11">
-        <v>1.4301999999999999</v>
+        <v>1.8223</v>
       </c>
       <c r="AD17" s="11">
-        <v>0.73140000000000005</v>
+        <v>1.1234999999999999</v>
       </c>
       <c r="AE17" s="12">
-        <v>1.0467</v>
+        <v>1.6077999999999999</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.2">
@@ -2794,25 +4851,25 @@
         <v>25.91</v>
       </c>
       <c r="Y18" s="11">
-        <v>12.61</v>
+        <v>12.65</v>
       </c>
       <c r="Z18" s="11">
-        <v>-13.3</v>
+        <v>-13.26</v>
       </c>
       <c r="AA18" s="12">
-        <v>-0.51329999999999998</v>
+        <v>-0.51180000000000003</v>
       </c>
       <c r="AB18" s="11">
         <v>1.4147000000000001</v>
       </c>
       <c r="AC18" s="11">
-        <v>1.4668000000000001</v>
+        <v>1.4715</v>
       </c>
       <c r="AD18" s="11">
-        <v>5.21E-2</v>
+        <v>5.6800000000000003E-2</v>
       </c>
       <c r="AE18" s="12">
-        <v>3.6799999999999999E-2</v>
+        <v>4.0099999999999997E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.2">
@@ -2889,13 +4946,13 @@
         <v>4.34</v>
       </c>
       <c r="Y19" s="11">
-        <v>15.46</v>
+        <v>15.5</v>
       </c>
       <c r="Z19" s="11">
-        <v>11.12</v>
+        <v>11.16</v>
       </c>
       <c r="AA19" s="12">
-        <v>2.5621999999999998</v>
+        <v>2.5714000000000001</v>
       </c>
       <c r="AB19" s="11">
         <v>0</v>
@@ -2972,37 +5029,37 @@
         <v>328.85</v>
       </c>
       <c r="U20" s="11">
-        <v>126.73</v>
+        <v>126.17</v>
       </c>
       <c r="V20" s="11">
-        <v>-202.12</v>
+        <v>-202.68</v>
       </c>
       <c r="W20" s="12">
-        <v>-0.61460000000000004</v>
+        <v>-0.61629999999999996</v>
       </c>
       <c r="X20" s="11">
         <v>353.8</v>
       </c>
       <c r="Y20" s="11">
-        <v>216.24</v>
+        <v>219.62</v>
       </c>
       <c r="Z20" s="11">
-        <v>-137.56</v>
+        <v>-134.18</v>
       </c>
       <c r="AA20" s="12">
-        <v>-0.38879999999999998</v>
+        <v>-0.37930000000000003</v>
       </c>
       <c r="AB20" s="11">
         <v>1.8688</v>
       </c>
       <c r="AC20" s="11">
-        <v>0.36919999999999997</v>
+        <v>0.37190000000000001</v>
       </c>
       <c r="AD20" s="11">
-        <v>-1.4996</v>
+        <v>-1.4968999999999999</v>
       </c>
       <c r="AE20" s="12">
-        <v>-0.8024</v>
+        <v>-0.80100000000000005</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.2">
@@ -3055,10 +5112,10 @@
         <v>0</v>
       </c>
       <c r="Q21" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R21" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="S21" s="12">
         <v>1</v>
@@ -3067,10 +5124,10 @@
         <v>0</v>
       </c>
       <c r="U21" s="11">
-        <v>139</v>
+        <v>139.21</v>
       </c>
       <c r="V21" s="11">
-        <v>139</v>
+        <v>139.21</v>
       </c>
       <c r="W21" s="12">
         <v>1</v>
@@ -3079,25 +5136,25 @@
         <v>11.56</v>
       </c>
       <c r="Y21" s="11">
-        <v>59.85</v>
+        <v>66.790000000000006</v>
       </c>
       <c r="Z21" s="11">
-        <v>48.29</v>
+        <v>55.23</v>
       </c>
       <c r="AA21" s="12">
-        <v>4.1772999999999998</v>
+        <v>4.7777000000000003</v>
       </c>
       <c r="AB21" s="11">
         <v>0.31490000000000001</v>
       </c>
       <c r="AC21" s="11">
-        <v>1.4286000000000001</v>
+        <v>1.4336</v>
       </c>
       <c r="AD21" s="11">
-        <v>1.1136999999999999</v>
+        <v>1.1187</v>
       </c>
       <c r="AE21" s="12">
-        <v>3.5367000000000002</v>
+        <v>3.5526</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.2">
@@ -3174,13 +5231,13 @@
         <v>11.23</v>
       </c>
       <c r="Y22" s="11">
-        <v>10.14</v>
+        <v>10.210000000000001</v>
       </c>
       <c r="Z22" s="11">
-        <v>-1.0900000000000001</v>
+        <v>-1.02</v>
       </c>
       <c r="AA22" s="12">
-        <v>-9.7100000000000006E-2</v>
+        <v>-9.0800000000000006E-2</v>
       </c>
       <c r="AB22" s="11">
         <v>0</v>
@@ -3269,13 +5326,13 @@
         <v>11.9</v>
       </c>
       <c r="Y23" s="11">
-        <v>20.2</v>
+        <v>20.23</v>
       </c>
       <c r="Z23" s="11">
-        <v>8.3000000000000007</v>
+        <v>8.33</v>
       </c>
       <c r="AA23" s="12">
-        <v>0.69750000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="AB23" s="11">
         <v>0</v>
@@ -3542,25 +5599,25 @@
         <v>58.68</v>
       </c>
       <c r="U26" s="11">
-        <v>-0.1</v>
+        <v>-0.28999999999999998</v>
       </c>
       <c r="V26" s="11">
-        <v>-58.78</v>
+        <v>-58.97</v>
       </c>
       <c r="W26" s="12">
-        <v>-1.0017</v>
+        <v>-1.0048999999999999</v>
       </c>
       <c r="X26" s="11">
         <v>78.84</v>
       </c>
       <c r="Y26" s="11">
-        <v>48.79</v>
+        <v>53.4</v>
       </c>
       <c r="Z26" s="11">
-        <v>-30.05</v>
+        <v>-25.44</v>
       </c>
       <c r="AA26" s="12">
-        <v>-0.38119999999999998</v>
+        <v>-0.32269999999999999</v>
       </c>
       <c r="AB26" s="11">
         <v>0.5141</v>
@@ -3649,13 +5706,13 @@
         <v>46.3</v>
       </c>
       <c r="Y27" s="11">
-        <v>19.75</v>
+        <v>23.85</v>
       </c>
       <c r="Z27" s="11">
-        <v>-26.55</v>
+        <v>-22.45</v>
       </c>
       <c r="AA27" s="12">
-        <v>-0.57340000000000002</v>
+        <v>-0.4849</v>
       </c>
       <c r="AB27" s="11">
         <v>0</v>
@@ -3744,13 +5801,13 @@
         <v>3.09</v>
       </c>
       <c r="Y28" s="11">
-        <v>11.47</v>
+        <v>13.24</v>
       </c>
       <c r="Z28" s="11">
-        <v>8.3800000000000008</v>
+        <v>10.15</v>
       </c>
       <c r="AA28" s="12">
-        <v>2.7120000000000002</v>
+        <v>3.2848000000000002</v>
       </c>
       <c r="AB28" s="11">
         <v>0</v>
@@ -3803,61 +5860,61 @@
         <v>4</v>
       </c>
       <c r="M29" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N29" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="O29" s="12">
-        <v>-1</v>
+        <v>-0.75</v>
       </c>
       <c r="P29" s="11">
         <v>4</v>
       </c>
       <c r="Q29" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="S29" s="12">
-        <v>-1</v>
+        <v>-0.75</v>
       </c>
       <c r="T29" s="11">
         <v>175.1</v>
       </c>
       <c r="U29" s="11">
-        <v>0</v>
+        <v>20.6</v>
       </c>
       <c r="V29" s="11">
-        <v>-175.1</v>
+        <v>-154.5</v>
       </c>
       <c r="W29" s="12">
-        <v>-1</v>
+        <v>-0.88239999999999996</v>
       </c>
       <c r="X29" s="11">
         <v>215.39</v>
       </c>
       <c r="Y29" s="11">
-        <v>28.61</v>
+        <v>39.979999999999997</v>
       </c>
       <c r="Z29" s="11">
-        <v>-186.78</v>
+        <v>-175.41</v>
       </c>
       <c r="AA29" s="12">
-        <v>-0.86719999999999997</v>
+        <v>-0.81440000000000001</v>
       </c>
       <c r="AB29" s="11">
         <v>1.528</v>
       </c>
       <c r="AC29" s="11">
-        <v>2.7492999999999999</v>
+        <v>3.9302000000000001</v>
       </c>
       <c r="AD29" s="11">
-        <v>1.2213000000000001</v>
+        <v>2.4022000000000001</v>
       </c>
       <c r="AE29" s="12">
-        <v>0.79930000000000001</v>
+        <v>1.5721000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.2">
@@ -3922,37 +5979,37 @@
         <v>224.88</v>
       </c>
       <c r="U30" s="11">
-        <v>112.38</v>
+        <v>112.57</v>
       </c>
       <c r="V30" s="11">
-        <v>-112.5</v>
+        <v>-112.31</v>
       </c>
       <c r="W30" s="12">
-        <v>-0.50029999999999997</v>
+        <v>-0.49940000000000001</v>
       </c>
       <c r="X30" s="11">
         <v>227.28</v>
       </c>
       <c r="Y30" s="11">
-        <v>99.18</v>
+        <v>107.29</v>
       </c>
       <c r="Z30" s="11">
-        <v>-128.1</v>
+        <v>-119.99</v>
       </c>
       <c r="AA30" s="12">
-        <v>-0.56359999999999999</v>
+        <v>-0.52790000000000004</v>
       </c>
       <c r="AB30" s="11">
         <v>0.1235</v>
       </c>
       <c r="AC30" s="11">
-        <v>3.3443000000000001</v>
+        <v>3.3654000000000002</v>
       </c>
       <c r="AD30" s="11">
-        <v>3.2208000000000001</v>
+        <v>3.2418999999999998</v>
       </c>
       <c r="AE30" s="12">
-        <v>26.0794</v>
+        <v>26.2502</v>
       </c>
     </row>
     <row r="31" spans="1:31" x14ac:dyDescent="0.2">
@@ -3993,13 +6050,13 @@
         <v>7</v>
       </c>
       <c r="M31" s="11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N31" s="11">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="O31" s="12">
-        <v>-0.28570000000000001</v>
+        <v>0</v>
       </c>
       <c r="P31" s="11">
         <v>7</v>
@@ -4017,37 +6074,37 @@
         <v>212.51</v>
       </c>
       <c r="U31" s="11">
-        <v>132.76</v>
+        <v>185.33</v>
       </c>
       <c r="V31" s="11">
-        <v>-79.75</v>
+        <v>-27.18</v>
       </c>
       <c r="W31" s="12">
-        <v>-0.37530000000000002</v>
+        <v>-0.12790000000000001</v>
       </c>
       <c r="X31" s="11">
         <v>187.2</v>
       </c>
       <c r="Y31" s="11">
-        <v>122.51</v>
+        <v>126.07</v>
       </c>
       <c r="Z31" s="11">
-        <v>-64.69</v>
+        <v>-61.13</v>
       </c>
       <c r="AA31" s="12">
-        <v>-0.34560000000000002</v>
+        <v>-0.32650000000000001</v>
       </c>
       <c r="AB31" s="11">
         <v>0.79920000000000002</v>
       </c>
       <c r="AC31" s="11">
-        <v>1.4389000000000001</v>
+        <v>1.8523000000000001</v>
       </c>
       <c r="AD31" s="11">
-        <v>0.63970000000000005</v>
+        <v>1.0530999999999999</v>
       </c>
       <c r="AE31" s="12">
-        <v>0.8004</v>
+        <v>1.3177000000000001</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.2">
@@ -4088,13 +6145,13 @@
         <v>2</v>
       </c>
       <c r="M32" s="11">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N32" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O32" s="12">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="P32" s="11">
         <v>2</v>
@@ -4112,34 +6169,34 @@
         <v>49.3</v>
       </c>
       <c r="U32" s="11">
-        <v>62.71</v>
+        <v>99.07</v>
       </c>
       <c r="V32" s="11">
-        <v>13.41</v>
+        <v>49.77</v>
       </c>
       <c r="W32" s="12">
-        <v>0.27200000000000002</v>
+        <v>1.0095000000000001</v>
       </c>
       <c r="X32" s="11">
         <v>80.510000000000005</v>
       </c>
       <c r="Y32" s="11">
-        <v>65.56</v>
+        <v>71.16</v>
       </c>
       <c r="Z32" s="11">
-        <v>-14.95</v>
+        <v>-9.35</v>
       </c>
       <c r="AA32" s="12">
-        <v>-0.1857</v>
+        <v>-0.11609999999999999</v>
       </c>
       <c r="AB32" s="11">
         <v>0</v>
       </c>
       <c r="AC32" s="11">
-        <v>0.89339999999999997</v>
+        <v>0.89580000000000004</v>
       </c>
       <c r="AD32" s="11">
-        <v>0.89339999999999997</v>
+        <v>0.89580000000000004</v>
       </c>
       <c r="AE32" s="12">
         <v>1</v>
@@ -4207,25 +6264,25 @@
         <v>67.260000000000005</v>
       </c>
       <c r="U33" s="11">
-        <v>34.11</v>
+        <v>34.369999999999997</v>
       </c>
       <c r="V33" s="11">
-        <v>-33.15</v>
+        <v>-32.89</v>
       </c>
       <c r="W33" s="12">
-        <v>-0.4929</v>
+        <v>-0.48899999999999999</v>
       </c>
       <c r="X33" s="11">
         <v>73</v>
       </c>
       <c r="Y33" s="11">
-        <v>28.89</v>
+        <v>32.06</v>
       </c>
       <c r="Z33" s="11">
-        <v>-44.11</v>
+        <v>-40.94</v>
       </c>
       <c r="AA33" s="12">
-        <v>-0.60419999999999996</v>
+        <v>-0.56079999999999997</v>
       </c>
       <c r="AB33" s="11">
         <v>3.1848999999999998</v>
@@ -4314,13 +6371,13 @@
         <v>63.59</v>
       </c>
       <c r="Y34" s="11">
-        <v>104.69</v>
+        <v>132.61000000000001</v>
       </c>
       <c r="Z34" s="11">
-        <v>41.1</v>
+        <v>69.02</v>
       </c>
       <c r="AA34" s="12">
-        <v>0.64629999999999999</v>
+        <v>1.0853999999999999</v>
       </c>
       <c r="AB34" s="11">
         <v>0</v>
@@ -4504,25 +6561,25 @@
         <v>303.52999999999997</v>
       </c>
       <c r="Y36" s="11">
-        <v>64.94</v>
+        <v>64.989999999999995</v>
       </c>
       <c r="Z36" s="11">
-        <v>-238.59</v>
+        <v>-238.54</v>
       </c>
       <c r="AA36" s="12">
-        <v>-0.78610000000000002</v>
+        <v>-0.78590000000000004</v>
       </c>
       <c r="AB36" s="11">
         <v>4.0427</v>
       </c>
       <c r="AC36" s="11">
-        <v>7.7786</v>
+        <v>9.2260000000000009</v>
       </c>
       <c r="AD36" s="11">
-        <v>3.7359</v>
+        <v>5.1833</v>
       </c>
       <c r="AE36" s="12">
-        <v>0.92410000000000003</v>
+        <v>1.2821</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.2">
@@ -4599,13 +6656,13 @@
         <v>86.18</v>
       </c>
       <c r="Y37" s="11">
-        <v>119.74</v>
+        <v>145.55000000000001</v>
       </c>
       <c r="Z37" s="11">
-        <v>33.56</v>
+        <v>59.37</v>
       </c>
       <c r="AA37" s="12">
-        <v>0.38940000000000002</v>
+        <v>0.68889999999999996</v>
       </c>
       <c r="AB37" s="11">
         <v>0</v>
@@ -4694,13 +6751,13 @@
         <v>103.45</v>
       </c>
       <c r="Y38" s="11">
-        <v>8.83</v>
+        <v>10.45</v>
       </c>
       <c r="Z38" s="11">
-        <v>-94.62</v>
+        <v>-93</v>
       </c>
       <c r="AA38" s="12">
-        <v>-0.91459999999999997</v>
+        <v>-0.89900000000000002</v>
       </c>
       <c r="AB38" s="11">
         <v>3.3999999999999998E-3</v>
@@ -4801,13 +6858,13 @@
         <v>9.8100000000000007E-2</v>
       </c>
       <c r="AC39" s="11">
-        <v>0</v>
+        <v>0.1643</v>
       </c>
       <c r="AD39" s="11">
-        <v>-9.8100000000000007E-2</v>
+        <v>6.6199999999999995E-2</v>
       </c>
       <c r="AE39" s="12">
-        <v>-1</v>
+        <v>0.67479999999999996</v>
       </c>
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.2">
@@ -4884,13 +6941,13 @@
         <v>29.29</v>
       </c>
       <c r="Y40" s="11">
-        <v>18.170000000000002</v>
+        <v>23.88</v>
       </c>
       <c r="Z40" s="11">
-        <v>-11.12</v>
+        <v>-5.41</v>
       </c>
       <c r="AA40" s="12">
-        <v>-0.37969999999999998</v>
+        <v>-0.1847</v>
       </c>
       <c r="AB40" s="11">
         <v>0</v>
@@ -5169,13 +7226,13 @@
         <v>62.03</v>
       </c>
       <c r="Y43" s="11">
-        <v>8.52</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="Z43" s="11">
-        <v>-53.51</v>
+        <v>-53.49</v>
       </c>
       <c r="AA43" s="12">
-        <v>-0.86260000000000003</v>
+        <v>-0.86229999999999996</v>
       </c>
       <c r="AB43" s="11">
         <v>0</v>
@@ -5264,13 +7321,13 @@
         <v>44.35</v>
       </c>
       <c r="Y44" s="11">
-        <v>26.54</v>
+        <v>26.61</v>
       </c>
       <c r="Z44" s="11">
-        <v>-17.809999999999999</v>
+        <v>-17.739999999999998</v>
       </c>
       <c r="AA44" s="12">
-        <v>-0.40160000000000001</v>
+        <v>-0.4</v>
       </c>
       <c r="AB44" s="11">
         <v>0</v>
@@ -5347,37 +7404,37 @@
         <v>272.62</v>
       </c>
       <c r="U45" s="11">
-        <v>227.64</v>
+        <v>227.99</v>
       </c>
       <c r="V45" s="11">
-        <v>-44.98</v>
+        <v>-44.63</v>
       </c>
       <c r="W45" s="12">
-        <v>-0.16500000000000001</v>
+        <v>-0.16370000000000001</v>
       </c>
       <c r="X45" s="11">
         <v>156.13999999999999</v>
       </c>
       <c r="Y45" s="11">
-        <v>167.4</v>
+        <v>172.46</v>
       </c>
       <c r="Z45" s="11">
-        <v>11.26</v>
+        <v>16.32</v>
       </c>
       <c r="AA45" s="12">
-        <v>7.2099999999999997E-2</v>
+        <v>0.1045</v>
       </c>
       <c r="AB45" s="11">
         <v>0.2029</v>
       </c>
       <c r="AC45" s="11">
-        <v>0.4365</v>
+        <v>0.4375</v>
       </c>
       <c r="AD45" s="11">
-        <v>0.2336</v>
+        <v>0.2346</v>
       </c>
       <c r="AE45" s="12">
-        <v>1.1513</v>
+        <v>1.1561999999999999</v>
       </c>
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.2">
@@ -5454,13 +7511,13 @@
         <v>208.83</v>
       </c>
       <c r="Y46" s="11">
-        <v>28.49</v>
+        <v>42.88</v>
       </c>
       <c r="Z46" s="11">
-        <v>-180.34</v>
+        <v>-165.95</v>
       </c>
       <c r="AA46" s="12">
-        <v>-0.86360000000000003</v>
+        <v>-0.79469999999999996</v>
       </c>
       <c r="AB46" s="11">
         <v>0</v>
@@ -5644,13 +7701,13 @@
         <v>86.46</v>
       </c>
       <c r="Y48" s="11">
-        <v>28.41</v>
+        <v>33.9</v>
       </c>
       <c r="Z48" s="11">
-        <v>-58.05</v>
+        <v>-52.56</v>
       </c>
       <c r="AA48" s="12">
-        <v>-0.6714</v>
+        <v>-0.6079</v>
       </c>
       <c r="AB48" s="11">
         <v>0</v>
@@ -5783,7 +7840,7 @@
         <v>60</v>
       </c>
       <c r="H50" s="10" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="I50" s="22">
         <v>45736</v>
@@ -5798,13 +7855,13 @@
         <v>4</v>
       </c>
       <c r="M50" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N50" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="O50" s="12">
-        <v>-1</v>
+        <v>-0.75</v>
       </c>
       <c r="P50" s="11">
         <v>4</v>
@@ -5822,13 +7879,13 @@
         <v>133.03</v>
       </c>
       <c r="U50" s="11">
-        <v>0</v>
+        <v>20.48</v>
       </c>
       <c r="V50" s="11">
-        <v>-133.03</v>
+        <v>-112.55</v>
       </c>
       <c r="W50" s="12">
-        <v>-1</v>
+        <v>-0.84599999999999997</v>
       </c>
       <c r="X50" s="11">
         <v>131.56</v>
@@ -6024,13 +8081,13 @@
         <v>2.4500000000000002</v>
       </c>
       <c r="Y52" s="11">
-        <v>15.04</v>
+        <v>15.06</v>
       </c>
       <c r="Z52" s="11">
-        <v>12.59</v>
+        <v>12.61</v>
       </c>
       <c r="AA52" s="12">
-        <v>5.1387999999999998</v>
+        <v>5.1468999999999996</v>
       </c>
       <c r="AB52" s="11">
         <v>0</v>
@@ -6119,13 +8176,13 @@
         <v>13.82</v>
       </c>
       <c r="Y53" s="11">
-        <v>17.690000000000001</v>
+        <v>22.09</v>
       </c>
       <c r="Z53" s="11">
-        <v>3.87</v>
+        <v>8.27</v>
       </c>
       <c r="AA53" s="12">
-        <v>0.28000000000000003</v>
+        <v>0.59840000000000004</v>
       </c>
       <c r="AB53" s="11">
         <v>0</v>
@@ -6214,10 +8271,10 @@
         <v>0</v>
       </c>
       <c r="Y54" s="11">
-        <v>69.489999999999995</v>
+        <v>69.42</v>
       </c>
       <c r="Z54" s="11">
-        <v>69.489999999999995</v>
+        <v>69.42</v>
       </c>
       <c r="AA54" s="12">
         <v>1</v>
@@ -6309,10 +8366,10 @@
         <v>0</v>
       </c>
       <c r="Y55" s="11">
-        <v>45.5</v>
+        <v>47.98</v>
       </c>
       <c r="Z55" s="11">
-        <v>45.5</v>
+        <v>47.98</v>
       </c>
       <c r="AA55" s="12">
         <v>1</v>
@@ -6392,10 +8449,10 @@
         <v>0</v>
       </c>
       <c r="U56" s="11">
-        <v>20.22</v>
+        <v>20.37</v>
       </c>
       <c r="V56" s="11">
-        <v>20.22</v>
+        <v>20.37</v>
       </c>
       <c r="W56" s="12">
         <v>1</v>
@@ -6404,10 +8461,10 @@
         <v>0</v>
       </c>
       <c r="Y56" s="11">
-        <v>25.46</v>
+        <v>27.97</v>
       </c>
       <c r="Z56" s="11">
-        <v>25.46</v>
+        <v>27.97</v>
       </c>
       <c r="AA56" s="12">
         <v>1</v>
@@ -6499,10 +8556,10 @@
         <v>0</v>
       </c>
       <c r="Y57" s="11">
-        <v>20.6</v>
+        <v>22.36</v>
       </c>
       <c r="Z57" s="11">
-        <v>20.6</v>
+        <v>22.36</v>
       </c>
       <c r="AA57" s="12">
         <v>1</v>
@@ -6677,10 +8734,10 @@
         <v>0</v>
       </c>
       <c r="U59" s="11">
-        <v>75.849999999999994</v>
+        <v>76.040000000000006</v>
       </c>
       <c r="V59" s="11">
-        <v>75.849999999999994</v>
+        <v>76.040000000000006</v>
       </c>
       <c r="W59" s="12">
         <v>1</v>
@@ -6689,10 +8746,10 @@
         <v>0</v>
       </c>
       <c r="Y59" s="11">
-        <v>136.78</v>
+        <v>143.38</v>
       </c>
       <c r="Z59" s="11">
-        <v>136.78</v>
+        <v>143.38</v>
       </c>
       <c r="AA59" s="12">
         <v>1</v>
@@ -6701,10 +8758,10 @@
         <v>0</v>
       </c>
       <c r="AC59" s="11">
-        <v>1.1674</v>
+        <v>1.407</v>
       </c>
       <c r="AD59" s="11">
-        <v>1.1674</v>
+        <v>1.407</v>
       </c>
       <c r="AE59" s="12">
         <v>1</v>
@@ -6784,10 +8841,10 @@
         <v>0</v>
       </c>
       <c r="Y60" s="11">
-        <v>19.690000000000001</v>
+        <v>53.86</v>
       </c>
       <c r="Z60" s="11">
-        <v>19.690000000000001</v>
+        <v>53.86</v>
       </c>
       <c r="AA60" s="12">
         <v>1</v>
@@ -6879,10 +8936,10 @@
         <v>0</v>
       </c>
       <c r="Y61" s="11">
-        <v>63.6</v>
+        <v>67.16</v>
       </c>
       <c r="Z61" s="11">
-        <v>63.6</v>
+        <v>67.16</v>
       </c>
       <c r="AA61" s="12">
         <v>1</v>
@@ -6974,10 +9031,10 @@
         <v>0</v>
       </c>
       <c r="Y62" s="11">
-        <v>4.75</v>
+        <v>4.76</v>
       </c>
       <c r="Z62" s="11">
-        <v>4.75</v>
+        <v>4.76</v>
       </c>
       <c r="AA62" s="12">
         <v>1</v>
@@ -7021,13 +9078,13 @@
         <v>127</v>
       </c>
       <c r="I63" s="22">
-        <v>46006</v>
+        <v>46111</v>
       </c>
       <c r="J63" s="22">
-        <v>46023</v>
+        <v>46111</v>
       </c>
       <c r="K63" s="23" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="L63" s="11">
         <v>0</v>
@@ -7069,10 +9126,10 @@
         <v>0</v>
       </c>
       <c r="Y63" s="11">
-        <v>70.02</v>
+        <v>72.05</v>
       </c>
       <c r="Z63" s="11">
-        <v>70.02</v>
+        <v>72.05</v>
       </c>
       <c r="AA63" s="12">
         <v>1</v>
@@ -7128,10 +9185,10 @@
         <v>0</v>
       </c>
       <c r="M64" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N64" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O64" s="12">
         <v>1</v>
@@ -7140,10 +9197,10 @@
         <v>0</v>
       </c>
       <c r="Q64" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R64" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S64" s="12">
         <v>1</v>
@@ -7152,10 +9209,10 @@
         <v>0</v>
       </c>
       <c r="U64" s="11">
-        <v>121.31</v>
+        <v>142.31</v>
       </c>
       <c r="V64" s="11">
-        <v>121.31</v>
+        <v>142.31</v>
       </c>
       <c r="W64" s="12">
         <v>1</v>
@@ -7164,10 +9221,10 @@
         <v>0</v>
       </c>
       <c r="Y64" s="11">
-        <v>31.24</v>
+        <v>33.06</v>
       </c>
       <c r="Z64" s="11">
-        <v>31.24</v>
+        <v>33.06</v>
       </c>
       <c r="AA64" s="12">
         <v>1</v>
@@ -7223,10 +9280,10 @@
         <v>0</v>
       </c>
       <c r="M65" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N65" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O65" s="12">
         <v>1</v>
@@ -7235,10 +9292,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R65" s="11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S65" s="12">
         <v>1</v>
@@ -7247,10 +9304,10 @@
         <v>0</v>
       </c>
       <c r="U65" s="11">
-        <v>119.03</v>
+        <v>155.6</v>
       </c>
       <c r="V65" s="11">
-        <v>119.03</v>
+        <v>155.6</v>
       </c>
       <c r="W65" s="12">
         <v>1</v>
@@ -7259,10 +9316,10 @@
         <v>0</v>
       </c>
       <c r="Y65" s="11">
-        <v>9.92</v>
+        <v>15.45</v>
       </c>
       <c r="Z65" s="11">
-        <v>9.92</v>
+        <v>15.45</v>
       </c>
       <c r="AA65" s="12">
         <v>1</v>
@@ -7277,6 +9334,101 @@
         <v>0</v>
       </c>
       <c r="AE65" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:31" x14ac:dyDescent="0.2">
+      <c r="A66" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C66" s="10">
+        <v>2043</v>
+      </c>
+      <c r="D66" s="10">
+        <v>2856</v>
+      </c>
+      <c r="E66" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="F66" s="10">
+        <v>118069</v>
+      </c>
+      <c r="G66" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="H66" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I66" s="22">
+        <v>46105</v>
+      </c>
+      <c r="J66" s="22">
+        <v>46113</v>
+      </c>
+      <c r="K66" s="23" t="s">
+        <v>128</v>
+      </c>
+      <c r="L66" s="11">
+        <v>0</v>
+      </c>
+      <c r="M66" s="11">
+        <v>1</v>
+      </c>
+      <c r="N66" s="11">
+        <v>1</v>
+      </c>
+      <c r="O66" s="12">
+        <v>1</v>
+      </c>
+      <c r="P66" s="11">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="11">
+        <v>1</v>
+      </c>
+      <c r="R66" s="11">
+        <v>1</v>
+      </c>
+      <c r="S66" s="12">
+        <v>1</v>
+      </c>
+      <c r="T66" s="11">
+        <v>0</v>
+      </c>
+      <c r="U66" s="11">
+        <v>21.34</v>
+      </c>
+      <c r="V66" s="11">
+        <v>21.34</v>
+      </c>
+      <c r="W66" s="12">
+        <v>1</v>
+      </c>
+      <c r="X66" s="11">
+        <v>0</v>
+      </c>
+      <c r="Y66" s="11">
+        <v>1.78</v>
+      </c>
+      <c r="Z66" s="11">
+        <v>1.78</v>
+      </c>
+      <c r="AA66" s="12">
+        <v>1</v>
+      </c>
+      <c r="AB66" s="11">
+        <v>0</v>
+      </c>
+      <c r="AC66" s="11">
+        <v>0</v>
+      </c>
+      <c r="AD66" s="11">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="12">
         <v>0</v>
       </c>
     </row>
@@ -7288,37 +9440,312 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A7:C65">
-    <cfRule type="expression" dxfId="6" priority="29" stopIfTrue="1">
+  <conditionalFormatting sqref="AD7:AE66 N7:O66 R7:S66 V7:W66 Z7:AA66">
+    <cfRule type="cellIs" dxfId="61" priority="40" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:B66">
+    <cfRule type="expression" dxfId="60" priority="61" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:W65">
-    <cfRule type="expression" dxfId="5" priority="41" stopIfTrue="1">
+  <conditionalFormatting sqref="C7:C66">
+    <cfRule type="expression" dxfId="59" priority="60" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D7:V65">
-    <cfRule type="expression" dxfId="4" priority="10">
+  <conditionalFormatting sqref="D7:D66">
+    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N7:O65 R7:S65 V7:W65 Z7:AA65 AD7:AE65">
-    <cfRule type="cellIs" dxfId="3" priority="9" operator="lessThan">
+  <conditionalFormatting sqref="E7:E66">
+    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F66">
+    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:G66">
+    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H66">
+    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:I66">
+    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:J66">
+    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K66">
+    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:L66">
+    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7:M66">
+    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N66">
+    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O7:O66">
+    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:P66">
+    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q7:Q66">
+    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R66">
+    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S7:S66">
+    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T7:T66">
+    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:U66">
+    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V7:V66">
+    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:W66">
+    <cfRule type="expression" dxfId="39" priority="62" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X7:X66">
+    <cfRule type="expression" dxfId="38" priority="39" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Y66">
+    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z7:Z66">
+    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA7:AA66">
+    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB7:AB66">
+    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC7:AC66">
+    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD66">
+    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE7:AE66">
+    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AE66 N7:O66 R7:S66 V7:W66 Z7:AA66">
+    <cfRule type="cellIs" dxfId="30" priority="9" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V7:W65 Z7:AA65 AD7:AE65 N7:O65 R7:S65">
-    <cfRule type="cellIs" dxfId="2" priority="40" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:AE65">
-    <cfRule type="expression" dxfId="1" priority="31" stopIfTrue="1">
+  <conditionalFormatting sqref="A7:B66">
+    <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X7:AE65">
+  <conditionalFormatting sqref="C7:C66">
+    <cfRule type="expression" dxfId="28" priority="29" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:D66">
+    <cfRule type="expression" dxfId="27" priority="28">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E7:E66">
+    <cfRule type="expression" dxfId="26" priority="27">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F7:F66">
+    <cfRule type="expression" dxfId="25" priority="26">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:G66">
+    <cfRule type="expression" dxfId="24" priority="25">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H7:H66">
+    <cfRule type="expression" dxfId="23" priority="24">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I7:I66">
+    <cfRule type="expression" dxfId="22" priority="23">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J7:J66">
+    <cfRule type="expression" dxfId="21" priority="22">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K7:K66">
+    <cfRule type="expression" dxfId="20" priority="21">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L7:L66">
+    <cfRule type="expression" dxfId="19" priority="20">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M7:M66">
+    <cfRule type="expression" dxfId="18" priority="19">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:N66">
+    <cfRule type="expression" dxfId="17" priority="18">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O7:O66">
+    <cfRule type="expression" dxfId="16" priority="17">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P7:P66">
+    <cfRule type="expression" dxfId="15" priority="16">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q7:Q66">
+    <cfRule type="expression" dxfId="14" priority="15">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R66">
+    <cfRule type="expression" dxfId="13" priority="14">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S7:S66">
+    <cfRule type="expression" dxfId="12" priority="13">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T7:T66">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U7:U66">
+    <cfRule type="expression" dxfId="10" priority="11">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V7:V66">
+    <cfRule type="expression" dxfId="9" priority="10">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:W66">
+    <cfRule type="expression" dxfId="8" priority="31" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X7:X66">
+    <cfRule type="expression" dxfId="7" priority="8">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y7:Y66">
+    <cfRule type="expression" dxfId="6" priority="7">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z7:Z66">
+    <cfRule type="expression" dxfId="5" priority="6">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA7:AA66">
+    <cfRule type="expression" dxfId="4" priority="5">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB7:AB66">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC7:AC66">
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD7:AD66">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE7:AE66">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-15 13:01)
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8E8360-929D-C74A-BB41-15CF60D3ADB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99484549-DB6B-D94E-9138-9FD40A100275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="100" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>
@@ -677,2101 +677,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="136">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="double">
-          <color indexed="22"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="double">
-          <color indexed="22"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color indexed="9"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor indexed="18"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="double">
-          <color indexed="22"/>
-        </left>
-        <right style="double">
-          <color indexed="22"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="1" hidden="1"/>
-    </dxf>
+  <dxfs count="10">
     <dxf>
       <border>
         <left style="hair">
@@ -2898,6 +804,56 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="double">
+          <color indexed="22"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="double">
+          <color indexed="22"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color indexed="9"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor indexed="18"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="double">
+          <color indexed="22"/>
+        </left>
+        <right style="double">
+          <color indexed="22"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="1" hidden="1"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -2912,7 +868,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="128" headerRowBorderDxfId="126" tableBorderDxfId="127">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="9" headerRowBorderDxfId="8" tableBorderDxfId="7">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -9440,312 +7396,37 @@
     <mergeCell ref="X2:AA2"/>
     <mergeCell ref="AB2:AE2"/>
   </mergeCells>
-  <conditionalFormatting sqref="AD7:AE66 N7:O66 R7:S66 V7:W66 Z7:AA66">
-    <cfRule type="cellIs" dxfId="61" priority="40" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="A7:C66">
+    <cfRule type="expression" dxfId="6" priority="29" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A7:W66">
+    <cfRule type="expression" dxfId="5" priority="41" stopIfTrue="1">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7:V66">
+    <cfRule type="expression" dxfId="4" priority="10">
+      <formula>$B7&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N7:O66 R7:S66 V7:W66 Z7:AA66 AD7:AE66">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B66">
-    <cfRule type="expression" dxfId="60" priority="61" stopIfTrue="1">
+  <conditionalFormatting sqref="V7:W66 Z7:AA66 AD7:AE66 N7:O66 R7:S66">
+    <cfRule type="cellIs" dxfId="2" priority="40" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W7:AE66">
+    <cfRule type="expression" dxfId="1" priority="31" stopIfTrue="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C7:C66">
-    <cfRule type="expression" dxfId="59" priority="60" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D66">
-    <cfRule type="expression" dxfId="58" priority="59" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E66">
-    <cfRule type="expression" dxfId="57" priority="58" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F66">
-    <cfRule type="expression" dxfId="56" priority="57" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G66">
-    <cfRule type="expression" dxfId="55" priority="56" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H66">
-    <cfRule type="expression" dxfId="54" priority="55" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I66">
-    <cfRule type="expression" dxfId="53" priority="54" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J66">
-    <cfRule type="expression" dxfId="52" priority="53" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K66">
-    <cfRule type="expression" dxfId="51" priority="52" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L66">
-    <cfRule type="expression" dxfId="50" priority="51" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M66">
-    <cfRule type="expression" dxfId="49" priority="50" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N66">
-    <cfRule type="expression" dxfId="48" priority="49" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O7:O66">
-    <cfRule type="expression" dxfId="47" priority="48" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P66">
-    <cfRule type="expression" dxfId="46" priority="47" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q7:Q66">
-    <cfRule type="expression" dxfId="45" priority="46" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R7:R66">
-    <cfRule type="expression" dxfId="44" priority="45" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S66">
-    <cfRule type="expression" dxfId="43" priority="44" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T7:T66">
-    <cfRule type="expression" dxfId="42" priority="43" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U66">
-    <cfRule type="expression" dxfId="41" priority="42" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7:V66">
-    <cfRule type="expression" dxfId="40" priority="41" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:W66">
-    <cfRule type="expression" dxfId="39" priority="62" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X7:X66">
-    <cfRule type="expression" dxfId="38" priority="39" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Y66">
-    <cfRule type="expression" dxfId="37" priority="38" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z7:Z66">
-    <cfRule type="expression" dxfId="36" priority="37" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA66">
-    <cfRule type="expression" dxfId="35" priority="36" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB7:AB66">
-    <cfRule type="expression" dxfId="34" priority="35" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7:AC66">
-    <cfRule type="expression" dxfId="33" priority="34" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AD66">
-    <cfRule type="expression" dxfId="32" priority="33" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE7:AE66">
-    <cfRule type="expression" dxfId="31" priority="32" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AE66 N7:O66 R7:S66 V7:W66 Z7:AA66">
-    <cfRule type="cellIs" dxfId="30" priority="9" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A7:B66">
-    <cfRule type="expression" dxfId="29" priority="30" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7:C66">
-    <cfRule type="expression" dxfId="28" priority="29" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7:D66">
-    <cfRule type="expression" dxfId="27" priority="28">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7:E66">
-    <cfRule type="expression" dxfId="26" priority="27">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F7:F66">
-    <cfRule type="expression" dxfId="25" priority="26">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G66">
-    <cfRule type="expression" dxfId="24" priority="25">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H66">
-    <cfRule type="expression" dxfId="23" priority="24">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I66">
-    <cfRule type="expression" dxfId="22" priority="23">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J66">
-    <cfRule type="expression" dxfId="21" priority="22">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7:K66">
-    <cfRule type="expression" dxfId="20" priority="21">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L7:L66">
-    <cfRule type="expression" dxfId="19" priority="20">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M7:M66">
-    <cfRule type="expression" dxfId="18" priority="19">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N7:N66">
-    <cfRule type="expression" dxfId="17" priority="18">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O7:O66">
-    <cfRule type="expression" dxfId="16" priority="17">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P7:P66">
-    <cfRule type="expression" dxfId="15" priority="16">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q7:Q66">
-    <cfRule type="expression" dxfId="14" priority="15">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R7:R66">
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S7:S66">
-    <cfRule type="expression" dxfId="12" priority="13">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T7:T66">
-    <cfRule type="expression" dxfId="11" priority="12">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U7:U66">
-    <cfRule type="expression" dxfId="10" priority="11">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V7:V66">
-    <cfRule type="expression" dxfId="9" priority="10">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W7:W66">
-    <cfRule type="expression" dxfId="8" priority="31" stopIfTrue="1">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X7:X66">
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Y7:Y66">
-    <cfRule type="expression" dxfId="6" priority="7">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z7:Z66">
-    <cfRule type="expression" dxfId="5" priority="6">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AA7:AA66">
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB7:AB66">
-    <cfRule type="expression" dxfId="3" priority="4">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC7:AC66">
-    <cfRule type="expression" dxfId="2" priority="3">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD7:AD66">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$B7&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE7:AE66">
+  <conditionalFormatting sqref="X7:AE66">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$B7&lt;&gt;""</formula>
     </cfRule>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-15 13:29)
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99484549-DB6B-D94E-9138-9FD40A100275}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07C41DBC-0F85-2547-AD45-E499275A69B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-20 11:05)
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DBB7603-FB08-1E41-86E5-4FB497F2845E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4E8461-310D-5344-AC16-5637620BBD14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
+    <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" activeTab="1" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
   <sheets>
     <sheet name="promotoria" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-13 11:06)
</commit_message>
<xml_diff>
--- a/administrador/comparativo_vida/comparativo vida.xlsx
+++ b/administrador/comparativo_vida/comparativo vida.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/administrador/comparativo_vida/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925BE45E-FFF4-F940-8C22-AC81EADFF646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{394FF3AD-AD04-C94A-992D-83E80F97060C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16320" xr2:uid="{E1D9733C-3B37-8B4F-9120-34426D0B6D20}"/>
   </bookViews>
@@ -672,14 +672,6 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
@@ -693,13 +685,21 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="72">
+  <dxfs count="136">
     <dxf>
       <border>
         <left style="hair">
@@ -1707,17 +1707,1181 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="double">
+          <color indexed="22"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
         <bottom style="double">
           <color indexed="22"/>
         </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="double">
-          <color indexed="22"/>
-        </top>
       </border>
     </dxf>
     <dxf>
@@ -1756,132 +2920,6 @@
       </border>
       <protection locked="1" hidden="1"/>
     </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1896,7 +2934,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="64" headerRowBorderDxfId="62" tableBorderDxfId="63">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5CEA801B-A74C-1349-A3D4-C6A1109DE591}" name="Tabla10" displayName="Tabla10" ref="A3:P5" totalsRowShown="0" headerRowDxfId="135" headerRowBorderDxfId="134" tableBorderDxfId="133">
   <autoFilter ref="A3:P5" xr:uid="{A29DCA76-5097-2F45-94DA-4B121F22F1F5}"/>
   <tableColumns count="16">
     <tableColumn id="1" xr3:uid="{A2D27468-D390-E245-85A6-B90C4BDF0CE1}" name="Polizas_Pagadas_Año_Anterior"/>
@@ -2245,7 +3283,7 @@
   <sheetData>
     <row r="1" spans="1:16" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="1">
-        <v>46136</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="46" thickBot="1" x14ac:dyDescent="0.25">
@@ -2321,25 +3359,25 @@
         <v>168</v>
       </c>
       <c r="B5" s="15">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="C5" s="15">
-        <v>-82</v>
+        <v>-67</v>
       </c>
       <c r="D5" s="16">
-        <v>-0.48809523809523814</v>
+        <v>-0.39880952380952384</v>
       </c>
       <c r="E5" s="15">
         <v>8098.38</v>
       </c>
       <c r="F5" s="15">
-        <v>4179.3500000000004</v>
+        <v>4768.13</v>
       </c>
       <c r="G5" s="15">
-        <v>-3919.03</v>
+        <v>-3330.25</v>
       </c>
       <c r="H5" s="16">
-        <v>-0.48392764972747637</v>
+        <v>-0.41122422015267246</v>
       </c>
       <c r="I5" s="15">
         <v>3</v>
@@ -2357,13 +3395,13 @@
         <v>372.32</v>
       </c>
       <c r="N5" s="15">
-        <v>106.9436</v>
+        <v>142.24350000000001</v>
       </c>
       <c r="O5" s="15">
-        <v>-265.37639999999999</v>
+        <v>-230.07650000000001</v>
       </c>
       <c r="P5" s="16">
-        <v>-0.7127642887838419</v>
+        <v>-0.61795364202836267</v>
       </c>
     </row>
   </sheetData>
@@ -2385,40 +3423,40 @@
   <sheetData>
     <row r="1" spans="1:31" ht="33" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1">
-        <v>46136</v>
+        <v>46142</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="L2" s="24" t="s">
+      <c r="L2" s="28" t="s">
         <v>75</v>
       </c>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="25" t="s">
+      <c r="M2" s="28"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-      <c r="S2" s="25"/>
-      <c r="T2" s="24" t="s">
+      <c r="Q2" s="29"/>
+      <c r="R2" s="29"/>
+      <c r="S2" s="29"/>
+      <c r="T2" s="28" t="s">
         <v>77</v>
       </c>
-      <c r="U2" s="24"/>
-      <c r="V2" s="24"/>
-      <c r="W2" s="24"/>
-      <c r="X2" s="25" t="s">
+      <c r="U2" s="28"/>
+      <c r="V2" s="28"/>
+      <c r="W2" s="28"/>
+      <c r="X2" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="Y2" s="25"/>
-      <c r="Z2" s="25"/>
-      <c r="AA2" s="25"/>
-      <c r="AB2" s="24" t="s">
+      <c r="Y2" s="29"/>
+      <c r="Z2" s="29"/>
+      <c r="AA2" s="29"/>
+      <c r="AB2" s="28" t="s">
         <v>79</v>
       </c>
-      <c r="AC2" s="24"/>
-      <c r="AD2" s="24"/>
-      <c r="AE2" s="24"/>
+      <c r="AC2" s="28"/>
+      <c r="AD2" s="28"/>
+      <c r="AE2" s="28"/>
     </row>
     <row r="3" spans="1:31" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -2548,38 +3586,38 @@
       <c r="AD4" s="13"/>
       <c r="AE4" s="20"/>
     </row>
-    <row r="5" spans="1:31" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="26"/>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="27"/>
-      <c r="M5" s="27"/>
-      <c r="N5" s="27"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="28"/>
-      <c r="T5" s="27"/>
-      <c r="U5" s="27"/>
-      <c r="V5" s="27"/>
-      <c r="W5" s="28"/>
-      <c r="X5" s="27"/>
-      <c r="Y5" s="27"/>
-      <c r="Z5" s="27"/>
-      <c r="AA5" s="28"/>
-      <c r="AB5" s="27"/>
-      <c r="AC5" s="27"/>
-      <c r="AD5" s="27"/>
-      <c r="AE5" s="28"/>
+    <row r="5" spans="1:31" s="27" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="24"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
+      <c r="H5" s="24"/>
+      <c r="I5" s="24"/>
+      <c r="J5" s="24"/>
+      <c r="K5" s="24"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="25"/>
+      <c r="O5" s="26"/>
+      <c r="P5" s="25"/>
+      <c r="Q5" s="25"/>
+      <c r="R5" s="25"/>
+      <c r="S5" s="26"/>
+      <c r="T5" s="25"/>
+      <c r="U5" s="25"/>
+      <c r="V5" s="25"/>
+      <c r="W5" s="26"/>
+      <c r="X5" s="25"/>
+      <c r="Y5" s="25"/>
+      <c r="Z5" s="25"/>
+      <c r="AA5" s="26"/>
+      <c r="AB5" s="25"/>
+      <c r="AC5" s="25"/>
+      <c r="AD5" s="25"/>
+      <c r="AE5" s="26"/>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
@@ -2738,37 +3776,37 @@
         <v>278.72000000000003</v>
       </c>
       <c r="U7" s="11">
-        <v>186.68</v>
+        <v>186.97</v>
       </c>
       <c r="V7" s="11">
-        <v>-92.04</v>
+        <v>-91.75</v>
       </c>
       <c r="W7" s="12">
-        <v>-0.33019999999999999</v>
+        <v>-0.32919999999999999</v>
       </c>
       <c r="X7" s="11">
         <v>326.55</v>
       </c>
       <c r="Y7" s="11">
-        <v>215.54</v>
+        <v>221.78</v>
       </c>
       <c r="Z7" s="11">
-        <v>-111.01</v>
+        <v>-104.77</v>
       </c>
       <c r="AA7" s="12">
-        <v>-0.33989999999999998</v>
+        <v>-0.32079999999999997</v>
       </c>
       <c r="AB7" s="11">
         <v>8.8199000000000005</v>
       </c>
       <c r="AC7" s="11">
-        <v>17.076799999999999</v>
+        <v>17.4192</v>
       </c>
       <c r="AD7" s="11">
-        <v>8.2568999999999999</v>
+        <v>8.5992999999999995</v>
       </c>
       <c r="AE7" s="12">
-        <v>0.93620000000000003</v>
+        <v>0.97499999999999998</v>
       </c>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.2">
@@ -3035,22 +4073,22 @@
         <v>31.17</v>
       </c>
       <c r="Y10" s="11">
-        <v>33.700000000000003</v>
+        <v>34.75</v>
       </c>
       <c r="Z10" s="11">
-        <v>2.5299999999999998</v>
+        <v>3.58</v>
       </c>
       <c r="AA10" s="12">
-        <v>8.1199999999999994E-2</v>
+        <v>0.1149</v>
       </c>
       <c r="AB10" s="11">
         <v>0</v>
       </c>
       <c r="AC10" s="11">
-        <v>0.2135</v>
+        <v>0.2147</v>
       </c>
       <c r="AD10" s="11">
-        <v>0.2135</v>
+        <v>0.2147</v>
       </c>
       <c r="AE10" s="12">
         <v>1</v>
@@ -3189,61 +4227,61 @@
         <v>13</v>
       </c>
       <c r="M12" s="11">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N12" s="11">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="O12" s="12">
-        <v>-7.6899999999999996E-2</v>
+        <v>7.6899999999999996E-2</v>
       </c>
       <c r="P12" s="11">
         <v>12</v>
       </c>
       <c r="Q12" s="11">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="R12" s="11">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="S12" s="12">
-        <v>-0.25</v>
+        <v>0</v>
       </c>
       <c r="T12" s="11">
         <v>619.97</v>
       </c>
       <c r="U12" s="11">
-        <v>570.01</v>
+        <v>701.65</v>
       </c>
       <c r="V12" s="11">
-        <v>-49.96</v>
+        <v>81.680000000000007</v>
       </c>
       <c r="W12" s="12">
-        <v>-8.0600000000000005E-2</v>
+        <v>0.13170000000000001</v>
       </c>
       <c r="X12" s="11">
         <v>876.03</v>
       </c>
       <c r="Y12" s="11">
-        <v>394.8</v>
+        <v>556.61</v>
       </c>
       <c r="Z12" s="11">
-        <v>-481.23</v>
+        <v>-319.42</v>
       </c>
       <c r="AA12" s="12">
-        <v>-0.54930000000000001</v>
+        <v>-0.36459999999999998</v>
       </c>
       <c r="AB12" s="11">
         <v>11.831099999999999</v>
       </c>
       <c r="AC12" s="11">
-        <v>21.471900000000002</v>
+        <v>21.480399999999999</v>
       </c>
       <c r="AD12" s="11">
-        <v>9.6408000000000005</v>
+        <v>9.6493000000000002</v>
       </c>
       <c r="AE12" s="12">
-        <v>0.81489999999999996</v>
+        <v>0.81559999999999999</v>
       </c>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
@@ -3320,25 +4358,25 @@
         <v>116.4</v>
       </c>
       <c r="Y13" s="11">
-        <v>44.91</v>
+        <v>49.3</v>
       </c>
       <c r="Z13" s="11">
-        <v>-71.489999999999995</v>
+        <v>-67.099999999999994</v>
       </c>
       <c r="AA13" s="12">
-        <v>-0.61419999999999997</v>
+        <v>-0.57650000000000001</v>
       </c>
       <c r="AB13" s="11">
         <v>6.7163000000000004</v>
       </c>
       <c r="AC13" s="11">
-        <v>8.6708999999999996</v>
+        <v>8.7853999999999992</v>
       </c>
       <c r="AD13" s="11">
-        <v>1.9545999999999999</v>
+        <v>2.0691000000000002</v>
       </c>
       <c r="AE13" s="12">
-        <v>0.29099999999999998</v>
+        <v>0.30809999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
@@ -3664,61 +4702,61 @@
         <v>7</v>
       </c>
       <c r="M17" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N17" s="11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O17" s="12">
-        <v>0.71430000000000005</v>
+        <v>0.85709999999999997</v>
       </c>
       <c r="P17" s="11">
         <v>8</v>
       </c>
       <c r="Q17" s="11">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R17" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S17" s="12">
-        <v>0.5</v>
+        <v>0.625</v>
       </c>
       <c r="T17" s="11">
         <v>1032.33</v>
       </c>
       <c r="U17" s="11">
-        <v>788.19</v>
+        <v>864.93</v>
       </c>
       <c r="V17" s="11">
-        <v>-244.14</v>
+        <v>-167.4</v>
       </c>
       <c r="W17" s="12">
-        <v>-0.23649999999999999</v>
+        <v>-0.16220000000000001</v>
       </c>
       <c r="X17" s="11">
         <v>820.67</v>
       </c>
       <c r="Y17" s="11">
-        <v>941.95</v>
+        <v>1050.1300000000001</v>
       </c>
       <c r="Z17" s="11">
-        <v>121.28</v>
+        <v>229.46</v>
       </c>
       <c r="AA17" s="12">
-        <v>0.14779999999999999</v>
+        <v>0.27960000000000002</v>
       </c>
       <c r="AB17" s="11">
         <v>1.9245000000000001</v>
       </c>
       <c r="AC17" s="11">
-        <v>4.5960000000000001</v>
+        <v>4.6641000000000004</v>
       </c>
       <c r="AD17" s="11">
-        <v>2.6715</v>
+        <v>2.7395999999999998</v>
       </c>
       <c r="AE17" s="12">
-        <v>1.3882000000000001</v>
+        <v>1.4235</v>
       </c>
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.2">
@@ -3771,49 +4809,49 @@
         <v>1</v>
       </c>
       <c r="Q18" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" s="11">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="S18" s="12">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T18" s="11">
         <v>19.260000000000002</v>
       </c>
       <c r="U18" s="11">
-        <v>41.45</v>
+        <v>41.68</v>
       </c>
       <c r="V18" s="11">
-        <v>22.19</v>
+        <v>22.42</v>
       </c>
       <c r="W18" s="12">
-        <v>1.1520999999999999</v>
+        <v>1.1640999999999999</v>
       </c>
       <c r="X18" s="11">
         <v>29.28</v>
       </c>
       <c r="Y18" s="11">
-        <v>16.89</v>
+        <v>20.39</v>
       </c>
       <c r="Z18" s="11">
-        <v>-12.39</v>
+        <v>-8.89</v>
       </c>
       <c r="AA18" s="12">
-        <v>-0.42320000000000002</v>
+        <v>-0.30359999999999998</v>
       </c>
       <c r="AB18" s="11">
         <v>2.0203000000000002</v>
       </c>
       <c r="AC18" s="11">
-        <v>2.1012</v>
+        <v>2.1046999999999998</v>
       </c>
       <c r="AD18" s="11">
-        <v>8.09E-2</v>
+        <v>8.4400000000000003E-2</v>
       </c>
       <c r="AE18" s="12">
-        <v>0.04</v>
+        <v>4.1799999999999997E-2</v>
       </c>
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.2">
@@ -3890,13 +4928,13 @@
         <v>6.52</v>
       </c>
       <c r="Y19" s="11">
-        <v>20.7</v>
+        <v>20.73</v>
       </c>
       <c r="Z19" s="11">
-        <v>14.18</v>
+        <v>14.21</v>
       </c>
       <c r="AA19" s="12">
-        <v>2.1747999999999998</v>
+        <v>2.1793999999999998</v>
       </c>
       <c r="AB19" s="11">
         <v>0</v>
@@ -3949,61 +4987,61 @@
         <v>11</v>
       </c>
       <c r="M20" s="11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N20" s="11">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="O20" s="12">
-        <v>-0.2727</v>
+        <v>-0.18179999999999999</v>
       </c>
       <c r="P20" s="11">
         <v>11</v>
       </c>
       <c r="Q20" s="11">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="R20" s="11">
-        <v>-7</v>
+        <v>-3</v>
       </c>
       <c r="S20" s="12">
-        <v>-0.63639999999999997</v>
+        <v>-0.2727</v>
       </c>
       <c r="T20" s="11">
         <v>429.71</v>
       </c>
       <c r="U20" s="11">
-        <v>360.76</v>
+        <v>407.52</v>
       </c>
       <c r="V20" s="11">
-        <v>-68.95</v>
+        <v>-22.19</v>
       </c>
       <c r="W20" s="12">
-        <v>-0.1605</v>
+        <v>-5.16E-2</v>
       </c>
       <c r="X20" s="11">
         <v>513.05999999999995</v>
       </c>
       <c r="Y20" s="11">
-        <v>243.25</v>
+        <v>393.63</v>
       </c>
       <c r="Z20" s="11">
-        <v>-269.81</v>
+        <v>-119.43</v>
       </c>
       <c r="AA20" s="12">
-        <v>-0.52590000000000003</v>
+        <v>-0.23280000000000001</v>
       </c>
       <c r="AB20" s="11">
         <v>1.8688</v>
       </c>
       <c r="AC20" s="11">
-        <v>0.62990000000000002</v>
+        <v>1.544</v>
       </c>
       <c r="AD20" s="11">
-        <v>-1.2388999999999999</v>
+        <v>-0.32479999999999998</v>
       </c>
       <c r="AE20" s="12">
-        <v>-0.66290000000000004</v>
+        <v>-0.17380000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.2">
@@ -4080,25 +5118,25 @@
         <v>15.44</v>
       </c>
       <c r="Y21" s="11">
-        <v>69.099999999999994</v>
+        <v>73.78</v>
       </c>
       <c r="Z21" s="11">
-        <v>53.66</v>
+        <v>58.34</v>
       </c>
       <c r="AA21" s="12">
-        <v>3.4754</v>
+        <v>3.7785000000000002</v>
       </c>
       <c r="AB21" s="11">
         <v>0.42049999999999998</v>
       </c>
       <c r="AC21" s="11">
-        <v>5.0438999999999998</v>
+        <v>5.0641999999999996</v>
       </c>
       <c r="AD21" s="11">
-        <v>4.6234000000000002</v>
+        <v>4.6436999999999999</v>
       </c>
       <c r="AE21" s="12">
-        <v>10.994999999999999</v>
+        <v>11.0433</v>
       </c>
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.2">
@@ -4270,10 +5308,10 @@
         <v>1468.63</v>
       </c>
       <c r="Y23" s="11">
-        <v>24.11</v>
+        <v>24.14</v>
       </c>
       <c r="Z23" s="11">
-        <v>-1444.52</v>
+        <v>-1444.49</v>
       </c>
       <c r="AA23" s="12">
         <v>-0.98360000000000003</v>
@@ -4555,25 +5593,25 @@
         <v>85.04</v>
       </c>
       <c r="Y26" s="11">
-        <v>59.82</v>
+        <v>68.03</v>
       </c>
       <c r="Z26" s="11">
-        <v>-25.22</v>
+        <v>-17.010000000000002</v>
       </c>
       <c r="AA26" s="12">
-        <v>-0.29659999999999997</v>
+        <v>-0.2</v>
       </c>
       <c r="AB26" s="11">
         <v>0.68210000000000004</v>
       </c>
       <c r="AC26" s="11">
-        <v>0.81779999999999997</v>
+        <v>1.4392</v>
       </c>
       <c r="AD26" s="11">
-        <v>0.13569999999999999</v>
+        <v>0.7571</v>
       </c>
       <c r="AE26" s="12">
-        <v>0.19889999999999999</v>
+        <v>1.1100000000000001</v>
       </c>
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.2">
@@ -4650,13 +5688,13 @@
         <v>51.12</v>
       </c>
       <c r="Y27" s="11">
-        <v>28.57</v>
+        <v>32.700000000000003</v>
       </c>
       <c r="Z27" s="11">
-        <v>-22.55</v>
+        <v>-18.420000000000002</v>
       </c>
       <c r="AA27" s="12">
-        <v>-0.44109999999999999</v>
+        <v>-0.36030000000000001</v>
       </c>
       <c r="AB27" s="11">
         <v>0</v>
@@ -4733,10 +5771,10 @@
         <v>0</v>
       </c>
       <c r="U28" s="11">
-        <v>30.56</v>
+        <v>30.73</v>
       </c>
       <c r="V28" s="11">
-        <v>30.56</v>
+        <v>30.73</v>
       </c>
       <c r="W28" s="12">
         <v>1</v>
@@ -4745,13 +5783,13 @@
         <v>3.09</v>
       </c>
       <c r="Y28" s="11">
-        <v>13.24</v>
+        <v>21.33</v>
       </c>
       <c r="Z28" s="11">
-        <v>10.15</v>
+        <v>18.239999999999998</v>
       </c>
       <c r="AA28" s="12">
-        <v>3.2848000000000002</v>
+        <v>5.9028999999999998</v>
       </c>
       <c r="AB28" s="11">
         <v>0</v>
@@ -4828,37 +5866,37 @@
         <v>236.49</v>
       </c>
       <c r="U29" s="11">
-        <v>50.28</v>
+        <v>50.45</v>
       </c>
       <c r="V29" s="11">
-        <v>-186.21</v>
+        <v>-186.04</v>
       </c>
       <c r="W29" s="12">
-        <v>-0.78739999999999999</v>
+        <v>-0.78669999999999995</v>
       </c>
       <c r="X29" s="11">
         <v>262.24</v>
       </c>
       <c r="Y29" s="11">
-        <v>47.63</v>
+        <v>48.72</v>
       </c>
       <c r="Z29" s="11">
-        <v>-214.61</v>
+        <v>-213.52</v>
       </c>
       <c r="AA29" s="12">
-        <v>-0.81840000000000002</v>
+        <v>-0.81420000000000003</v>
       </c>
       <c r="AB29" s="11">
         <v>1.8343</v>
       </c>
       <c r="AC29" s="11">
-        <v>4.8116000000000003</v>
+        <v>6.0392999999999999</v>
       </c>
       <c r="AD29" s="11">
-        <v>2.9773000000000001</v>
+        <v>4.2050000000000001</v>
       </c>
       <c r="AE29" s="12">
-        <v>1.6231</v>
+        <v>2.2924000000000002</v>
       </c>
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.2">
@@ -4935,13 +5973,13 @@
         <v>316.83999999999997</v>
       </c>
       <c r="Y30" s="11">
-        <v>117.91</v>
+        <v>119.71</v>
       </c>
       <c r="Z30" s="11">
-        <v>-198.93</v>
+        <v>-197.13</v>
       </c>
       <c r="AA30" s="12">
-        <v>-0.62790000000000001</v>
+        <v>-0.62219999999999998</v>
       </c>
       <c r="AB30" s="11">
         <v>0.1235</v>
@@ -5018,37 +6056,37 @@
         <v>260.14999999999998</v>
       </c>
       <c r="U31" s="11">
-        <v>185.33</v>
+        <v>160.13</v>
       </c>
       <c r="V31" s="11">
-        <v>-74.819999999999993</v>
+        <v>-100.02</v>
       </c>
       <c r="W31" s="12">
-        <v>-0.28760000000000002</v>
+        <v>-0.38450000000000001</v>
       </c>
       <c r="X31" s="11">
         <v>234.63</v>
       </c>
       <c r="Y31" s="11">
-        <v>159.33000000000001</v>
+        <v>159.51</v>
       </c>
       <c r="Z31" s="11">
-        <v>-75.3</v>
+        <v>-75.12</v>
       </c>
       <c r="AA31" s="12">
-        <v>-0.32090000000000002</v>
+        <v>-0.32019999999999998</v>
       </c>
       <c r="AB31" s="11">
         <v>1.0677000000000001</v>
       </c>
       <c r="AC31" s="11">
-        <v>2.2037</v>
+        <v>2.4571000000000001</v>
       </c>
       <c r="AD31" s="11">
-        <v>1.1359999999999999</v>
+        <v>1.3894</v>
       </c>
       <c r="AE31" s="12">
-        <v>1.0640000000000001</v>
+        <v>1.3012999999999999</v>
       </c>
     </row>
     <row r="32" spans="1:31" x14ac:dyDescent="0.2">
@@ -5089,58 +6127,58 @@
         <v>2</v>
       </c>
       <c r="M32" s="11">
+        <v>6</v>
+      </c>
+      <c r="N32" s="11">
         <v>4</v>
       </c>
-      <c r="N32" s="11">
+      <c r="O32" s="12">
         <v>2</v>
-      </c>
-      <c r="O32" s="12">
-        <v>1</v>
       </c>
       <c r="P32" s="11">
         <v>2</v>
       </c>
       <c r="Q32" s="11">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="R32" s="11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="S32" s="12">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="T32" s="11">
         <v>49.3</v>
       </c>
       <c r="U32" s="11">
-        <v>123.69</v>
+        <v>174.68</v>
       </c>
       <c r="V32" s="11">
-        <v>74.39</v>
+        <v>125.38</v>
       </c>
       <c r="W32" s="12">
-        <v>1.5088999999999999</v>
+        <v>2.5432000000000001</v>
       </c>
       <c r="X32" s="11">
         <v>89.3</v>
       </c>
       <c r="Y32" s="11">
-        <v>114.94</v>
+        <v>130.19</v>
       </c>
       <c r="Z32" s="11">
-        <v>25.64</v>
+        <v>40.89</v>
       </c>
       <c r="AA32" s="12">
-        <v>0.28710000000000002</v>
+        <v>0.45789999999999997</v>
       </c>
       <c r="AB32" s="11">
         <v>0</v>
       </c>
       <c r="AC32" s="11">
-        <v>1.2112000000000001</v>
+        <v>1.2130000000000001</v>
       </c>
       <c r="AD32" s="11">
-        <v>1.2112000000000001</v>
+        <v>1.2130000000000001</v>
       </c>
       <c r="AE32" s="12">
         <v>1</v>
@@ -5220,13 +6258,13 @@
         <v>73</v>
       </c>
       <c r="Y33" s="11">
-        <v>49.61</v>
+        <v>49.71</v>
       </c>
       <c r="Z33" s="11">
-        <v>-23.39</v>
+        <v>-23.29</v>
       </c>
       <c r="AA33" s="12">
-        <v>-0.32040000000000002</v>
+        <v>-0.31900000000000001</v>
       </c>
       <c r="AB33" s="11">
         <v>3.1848999999999998</v>
@@ -5315,13 +6353,13 @@
         <v>349.84</v>
       </c>
       <c r="Y34" s="11">
-        <v>155.65</v>
+        <v>159.78</v>
       </c>
       <c r="Z34" s="11">
-        <v>-194.19</v>
+        <v>-190.06</v>
       </c>
       <c r="AA34" s="12">
-        <v>-0.55510000000000004</v>
+        <v>-0.54330000000000001</v>
       </c>
       <c r="AB34" s="11">
         <v>0</v>
@@ -5505,25 +6543,25 @@
         <v>377.79</v>
       </c>
       <c r="Y36" s="11">
-        <v>72.89</v>
+        <v>74.88</v>
       </c>
       <c r="Z36" s="11">
-        <v>-304.89999999999998</v>
+        <v>-302.91000000000003</v>
       </c>
       <c r="AA36" s="12">
-        <v>-0.80710000000000004</v>
+        <v>-0.80179999999999996</v>
       </c>
       <c r="AB36" s="11">
         <v>5.3985000000000003</v>
       </c>
       <c r="AC36" s="11">
-        <v>9.2260000000000009</v>
+        <v>10.6434</v>
       </c>
       <c r="AD36" s="11">
-        <v>3.8275000000000001</v>
+        <v>5.2449000000000003</v>
       </c>
       <c r="AE36" s="12">
-        <v>0.70899999999999996</v>
+        <v>0.97150000000000003</v>
       </c>
     </row>
     <row r="37" spans="1:31" x14ac:dyDescent="0.2">
@@ -5600,13 +6638,13 @@
         <v>185.17</v>
       </c>
       <c r="Y37" s="11">
-        <v>153.1</v>
+        <v>153.13999999999999</v>
       </c>
       <c r="Z37" s="11">
-        <v>-32.07</v>
+        <v>-32.03</v>
       </c>
       <c r="AA37" s="12">
-        <v>-0.17319999999999999</v>
+        <v>-0.17299999999999999</v>
       </c>
       <c r="AB37" s="11">
         <v>0</v>
@@ -5802,13 +6840,13 @@
         <v>0.30480000000000002</v>
       </c>
       <c r="AC39" s="11">
-        <v>0.1643</v>
+        <v>0.38040000000000002</v>
       </c>
       <c r="AD39" s="11">
-        <v>-0.14050000000000001</v>
+        <v>7.5600000000000001E-2</v>
       </c>
       <c r="AE39" s="12">
-        <v>-0.46100000000000002</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="40" spans="1:31" x14ac:dyDescent="0.2">
@@ -5885,13 +6923,13 @@
         <v>43.61</v>
       </c>
       <c r="Y40" s="11">
-        <v>30.08</v>
+        <v>30.98</v>
       </c>
       <c r="Z40" s="11">
-        <v>-13.53</v>
+        <v>-12.63</v>
       </c>
       <c r="AA40" s="12">
-        <v>-0.31019999999999998</v>
+        <v>-0.28960000000000002</v>
       </c>
       <c r="AB40" s="11">
         <v>0</v>
@@ -6158,25 +7196,25 @@
         <v>17.11</v>
       </c>
       <c r="U43" s="11">
-        <v>-0.22</v>
+        <v>-0.38</v>
       </c>
       <c r="V43" s="11">
-        <v>-17.329999999999998</v>
+        <v>-17.489999999999998</v>
       </c>
       <c r="W43" s="12">
-        <v>-1.0128999999999999</v>
+        <v>-1.0222</v>
       </c>
       <c r="X43" s="11">
         <v>105.69</v>
       </c>
       <c r="Y43" s="11">
-        <v>14.37</v>
+        <v>14.4</v>
       </c>
       <c r="Z43" s="11">
-        <v>-91.32</v>
+        <v>-91.29</v>
       </c>
       <c r="AA43" s="12">
-        <v>-0.86399999999999999</v>
+        <v>-0.86380000000000001</v>
       </c>
       <c r="AB43" s="11">
         <v>0</v>
@@ -6265,13 +7303,13 @@
         <v>50.17</v>
       </c>
       <c r="Y44" s="11">
-        <v>35.53</v>
+        <v>35.58</v>
       </c>
       <c r="Z44" s="11">
-        <v>-14.64</v>
+        <v>-14.59</v>
       </c>
       <c r="AA44" s="12">
-        <v>-0.2918</v>
+        <v>-0.2908</v>
       </c>
       <c r="AB44" s="11">
         <v>0</v>
@@ -6324,13 +7362,13 @@
         <v>14</v>
       </c>
       <c r="M45" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N45" s="11">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="O45" s="12">
-        <v>-0.28570000000000001</v>
+        <v>-0.21429999999999999</v>
       </c>
       <c r="P45" s="11">
         <v>14</v>
@@ -6348,37 +7386,37 @@
         <v>446.24</v>
       </c>
       <c r="U45" s="11">
-        <v>301.42</v>
+        <v>335.91</v>
       </c>
       <c r="V45" s="11">
-        <v>-144.82</v>
+        <v>-110.33</v>
       </c>
       <c r="W45" s="12">
-        <v>-0.32450000000000001</v>
+        <v>-0.2472</v>
       </c>
       <c r="X45" s="11">
         <v>198.56</v>
       </c>
       <c r="Y45" s="11">
-        <v>241.16</v>
+        <v>243.51</v>
       </c>
       <c r="Z45" s="11">
-        <v>42.6</v>
+        <v>44.95</v>
       </c>
       <c r="AA45" s="12">
-        <v>0.2145</v>
+        <v>0.22639999999999999</v>
       </c>
       <c r="AB45" s="11">
         <v>0.2029</v>
       </c>
       <c r="AC45" s="11">
-        <v>1.087</v>
+        <v>1.0906</v>
       </c>
       <c r="AD45" s="11">
-        <v>0.8841</v>
+        <v>0.88770000000000004</v>
       </c>
       <c r="AE45" s="12">
-        <v>4.3573000000000004</v>
+        <v>4.3750999999999998</v>
       </c>
     </row>
     <row r="46" spans="1:31" x14ac:dyDescent="0.2">
@@ -6455,13 +7493,13 @@
         <v>276.66000000000003</v>
       </c>
       <c r="Y46" s="11">
-        <v>57.27</v>
+        <v>71.81</v>
       </c>
       <c r="Z46" s="11">
-        <v>-219.39</v>
+        <v>-204.85</v>
       </c>
       <c r="AA46" s="12">
-        <v>-0.79300000000000004</v>
+        <v>-0.74039999999999995</v>
       </c>
       <c r="AB46" s="11">
         <v>0</v>
@@ -6633,25 +7671,25 @@
         <v>169.31</v>
       </c>
       <c r="U48" s="11">
-        <v>61.75</v>
+        <v>62.1</v>
       </c>
       <c r="V48" s="11">
-        <v>-107.56</v>
+        <v>-107.21</v>
       </c>
       <c r="W48" s="12">
-        <v>-0.63529999999999998</v>
+        <v>-0.63319999999999999</v>
       </c>
       <c r="X48" s="11">
         <v>93.74</v>
       </c>
       <c r="Y48" s="11">
-        <v>95.65</v>
+        <v>101.47</v>
       </c>
       <c r="Z48" s="11">
-        <v>1.91</v>
+        <v>7.73</v>
       </c>
       <c r="AA48" s="12">
-        <v>2.0400000000000001E-2</v>
+        <v>8.2500000000000004E-2</v>
       </c>
       <c r="AB48" s="11">
         <v>0</v>
@@ -6835,13 +7873,13 @@
         <v>131.56</v>
       </c>
       <c r="Y50" s="11">
-        <v>1.8</v>
+        <v>1.81</v>
       </c>
       <c r="Z50" s="11">
-        <v>-129.76</v>
+        <v>-129.75</v>
       </c>
       <c r="AA50" s="12">
-        <v>-0.98629999999999995</v>
+        <v>-0.98619999999999997</v>
       </c>
       <c r="AB50" s="11">
         <v>0</v>
@@ -7025,22 +8063,22 @@
         <v>51.32</v>
       </c>
       <c r="Y52" s="11">
-        <v>16.809999999999999</v>
+        <v>16.82</v>
       </c>
       <c r="Z52" s="11">
-        <v>-34.51</v>
+        <v>-34.5</v>
       </c>
       <c r="AA52" s="12">
-        <v>-0.6724</v>
+        <v>-0.67230000000000001</v>
       </c>
       <c r="AB52" s="11">
         <v>0</v>
       </c>
       <c r="AC52" s="11">
-        <v>3.8157000000000001</v>
+        <v>3.8371</v>
       </c>
       <c r="AD52" s="11">
-        <v>3.8157000000000001</v>
+        <v>3.8371</v>
       </c>
       <c r="AE52" s="12">
         <v>1</v>
@@ -7120,25 +8158,25 @@
         <v>81.27</v>
       </c>
       <c r="Y53" s="11">
-        <v>26.65</v>
+        <v>31.26</v>
       </c>
       <c r="Z53" s="11">
-        <v>-54.62</v>
+        <v>-50.01</v>
       </c>
       <c r="AA53" s="12">
-        <v>-0.67210000000000003</v>
+        <v>-0.61539999999999995</v>
       </c>
       <c r="AB53" s="11">
         <v>0</v>
       </c>
       <c r="AC53" s="11">
-        <v>0</v>
+        <v>0.4395</v>
       </c>
       <c r="AD53" s="11">
-        <v>0</v>
+        <v>0.4395</v>
       </c>
       <c r="AE53" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:31" x14ac:dyDescent="0.2">
@@ -7310,13 +8348,13 @@
         <v>13.61</v>
       </c>
       <c r="Y55" s="11">
-        <v>79.680000000000007</v>
+        <v>79.69</v>
       </c>
       <c r="Z55" s="11">
-        <v>66.069999999999993</v>
+        <v>66.08</v>
       </c>
       <c r="AA55" s="12">
-        <v>4.8544999999999998</v>
+        <v>4.8552999999999997</v>
       </c>
       <c r="AB55" s="11">
         <v>0</v>
@@ -7393,10 +8431,10 @@
         <v>0</v>
       </c>
       <c r="U56" s="11">
-        <v>40.83</v>
+        <v>41.06</v>
       </c>
       <c r="V56" s="11">
-        <v>40.83</v>
+        <v>41.06</v>
       </c>
       <c r="W56" s="12">
         <v>1</v>
@@ -7405,10 +8443,10 @@
         <v>0</v>
       </c>
       <c r="Y56" s="11">
-        <v>71.260000000000005</v>
+        <v>80.680000000000007</v>
       </c>
       <c r="Z56" s="11">
-        <v>71.260000000000005</v>
+        <v>80.680000000000007</v>
       </c>
       <c r="AA56" s="12">
         <v>1</v>
@@ -7500,10 +8538,10 @@
         <v>0</v>
       </c>
       <c r="Y57" s="11">
-        <v>31.3</v>
+        <v>31.32</v>
       </c>
       <c r="Z57" s="11">
-        <v>31.3</v>
+        <v>31.32</v>
       </c>
       <c r="AA57" s="12">
         <v>1</v>
@@ -7595,10 +8633,10 @@
         <v>0</v>
       </c>
       <c r="Y58" s="11">
-        <v>22.36</v>
+        <v>24.06</v>
       </c>
       <c r="Z58" s="11">
-        <v>22.36</v>
+        <v>24.06</v>
       </c>
       <c r="AA58" s="12">
         <v>1</v>
@@ -7785,10 +8823,10 @@
         <v>0</v>
       </c>
       <c r="Y60" s="11">
-        <v>148.4</v>
+        <v>150.26</v>
       </c>
       <c r="Z60" s="11">
-        <v>148.4</v>
+        <v>150.26</v>
       </c>
       <c r="AA60" s="12">
         <v>1</v>
@@ -7797,10 +8835,10 @@
         <v>0</v>
       </c>
       <c r="AC60" s="11">
-        <v>2.3195000000000001</v>
+        <v>2.5602</v>
       </c>
       <c r="AD60" s="11">
-        <v>2.3195000000000001</v>
+        <v>2.5602</v>
       </c>
       <c r="AE60" s="12">
         <v>1</v>
@@ -7880,10 +8918,10 @@
         <v>0</v>
       </c>
       <c r="Y61" s="11">
-        <v>53.86</v>
+        <v>55.61</v>
       </c>
       <c r="Z61" s="11">
-        <v>53.86</v>
+        <v>55.61</v>
       </c>
       <c r="AA61" s="12">
         <v>1</v>
@@ -7975,10 +9013,10 @@
         <v>0</v>
       </c>
       <c r="Y62" s="11">
-        <v>73.959999999999994</v>
+        <v>89.29</v>
       </c>
       <c r="Z62" s="11">
-        <v>73.959999999999994</v>
+        <v>89.29</v>
       </c>
       <c r="AA62" s="12">
         <v>1</v>
@@ -8070,10 +9108,10 @@
         <v>0</v>
       </c>
       <c r="Y63" s="11">
-        <v>6.35</v>
+        <v>6.36</v>
       </c>
       <c r="Z63" s="11">
-        <v>6.35</v>
+        <v>6.36</v>
       </c>
       <c r="AA63" s="12">
         <v>1</v>
@@ -8165,10 +9203,10 @@
         <v>0</v>
       </c>
       <c r="Y64" s="11">
-        <v>72.05</v>
+        <v>74.08</v>
       </c>
       <c r="Z64" s="11">
-        <v>72.05</v>
+        <v>74.08</v>
       </c>
       <c r="AA64" s="12">
         <v>1</v>
@@ -8224,10 +9262,10 @@
         <v>0</v>
       </c>
       <c r="M65" s="11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N65" s="11">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O65" s="12">
         <v>1</v>
@@ -8236,10 +9274,10 @@
         <v>0</v>
       </c>
       <c r="Q65" s="11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R65" s="11">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="S65" s="12">
         <v>1</v>
@@ -8248,10 +9286,10 @@
         <v>0</v>
       </c>
       <c r="U65" s="11">
-        <v>168.39</v>
+        <v>193.8</v>
       </c>
       <c r="V65" s="11">
-        <v>168.39</v>
+        <v>193.8</v>
       </c>
       <c r="W65" s="12">
         <v>1</v>
@@ -8260,10 +9298,10 @@
         <v>0</v>
       </c>
       <c r="Y65" s="11">
-        <v>34.89</v>
+        <v>68.16</v>
       </c>
       <c r="Z65" s="11">
-        <v>34.89</v>
+        <v>68.16</v>
       </c>
       <c r="AA65" s="12">
         <v>1</v>
@@ -8331,10 +9369,10 @@
         <v>0</v>
       </c>
       <c r="Q66" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R66" s="11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S66" s="12">
         <v>1</v>
@@ -8343,10 +9381,10 @@
         <v>0</v>
       </c>
       <c r="U66" s="11">
-        <v>220.42</v>
+        <v>220.78</v>
       </c>
       <c r="V66" s="11">
-        <v>220.42</v>
+        <v>220.78</v>
       </c>
       <c r="W66" s="12">
         <v>1</v>
@@ -8355,10 +9393,10 @@
         <v>0</v>
       </c>
       <c r="Y66" s="11">
-        <v>25.97</v>
+        <v>33.94</v>
       </c>
       <c r="Z66" s="11">
-        <v>25.97</v>
+        <v>33.94</v>
       </c>
       <c r="AA66" s="12">
         <v>1</v>
@@ -8450,10 +9488,10 @@
         <v>0</v>
       </c>
       <c r="Y67" s="11">
-        <v>1.78</v>
+        <v>3.57</v>
       </c>
       <c r="Z67" s="11">
-        <v>1.78</v>
+        <v>3.57</v>
       </c>
       <c r="AA67" s="12">
         <v>1</v>

</xml_diff>